<commit_message>
Agregar sitios web vía Apollo y enlace al sitio en Vercel
- 101 sitios web más desde la búsqueda gratuita de organizaciones de
  Apollo (solo coincidencias exactas o probables): 166 de 224 empresas.
- README con el enlace al sitio publicado.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H1ZHr5EuMixHqUzfpFW6bc
</commit_message>
<xml_diff>
--- a/data/empresas_b_chile.xlsx
+++ b/data/empresas_b_chile.xlsx
@@ -768,7 +768,11 @@
       <c r="AI2" t="inlineStr"/>
       <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>http://www.10pines.com</t>
+        </is>
+      </c>
       <c r="AM2" t="inlineStr"/>
       <c r="AN2" t="inlineStr"/>
       <c r="AO2" t="inlineStr"/>
@@ -791,9 +795,13 @@
         </is>
       </c>
       <c r="AZ2" t="n">
-        <v>29</v>
-      </c>
-      <c r="BA2" t="inlineStr"/>
+        <v>36</v>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB2" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -868,7 +876,11 @@
       <c r="AI3" t="inlineStr"/>
       <c r="AJ3" t="inlineStr"/>
       <c r="AK3" t="inlineStr"/>
-      <c r="AL3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>http://www.3ina.com</t>
+        </is>
+      </c>
       <c r="AM3" t="inlineStr"/>
       <c r="AN3" t="inlineStr"/>
       <c r="AO3" t="inlineStr"/>
@@ -891,11 +903,11 @@
         </is>
       </c>
       <c r="AZ3" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA3" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net//find-a-b-corp/company/3ina-cosmetics</t>
+          <t>https://www.bcorporation.net//find-a-b-corp/company/3ina-cosmetics | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB3" t="inlineStr">
@@ -1284,7 +1296,11 @@
       <c r="AI6" t="inlineStr"/>
       <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="inlineStr"/>
-      <c r="AL6" t="inlineStr"/>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>http://www.abrantes.cl</t>
+        </is>
+      </c>
       <c r="AM6" t="inlineStr"/>
       <c r="AN6" t="inlineStr"/>
       <c r="AO6" t="inlineStr"/>
@@ -1307,11 +1323,11 @@
         </is>
       </c>
       <c r="AZ6" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA6" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/abrantes/ | https://www.portalfruticola.com/noticias/2010/07/21/chile-nueva-empresa-de-champinones-de-sutil-planea-doblar-produccion-en-cinco-anos | https://www.portalfruticola.com/?p=2512</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/abrantes/ | https://www.portalfruticola.com/noticias/2010/07/21/chile-nueva-empresa-de-champinones-de-sutil-planea-doblar-produccion-en-cinco-anos | https://www.portalfruticola.com/?p=2512 | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB6" t="inlineStr">
@@ -2438,7 +2454,11 @@
       <c r="AI15" t="inlineStr"/>
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr"/>
-      <c r="AL15" t="inlineStr"/>
+      <c r="AL15" t="inlineStr">
+        <is>
+          <t>http://www.algeiba.com</t>
+        </is>
+      </c>
       <c r="AM15" t="inlineStr"/>
       <c r="AN15" t="inlineStr"/>
       <c r="AO15" t="inlineStr"/>
@@ -2461,9 +2481,13 @@
         </is>
       </c>
       <c r="AZ15" t="n">
-        <v>29</v>
-      </c>
-      <c r="BA15" t="inlineStr"/>
+        <v>36</v>
+      </c>
+      <c r="BA15" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB15" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -2906,7 +2930,11 @@
       <c r="AI19" t="inlineStr"/>
       <c r="AJ19" t="inlineStr"/>
       <c r="AK19" t="inlineStr"/>
-      <c r="AL19" t="inlineStr"/>
+      <c r="AL19" t="inlineStr">
+        <is>
+          <t>http://www.argentinaonthego.com</t>
+        </is>
+      </c>
       <c r="AM19" t="inlineStr"/>
       <c r="AN19" t="inlineStr"/>
       <c r="AO19" t="inlineStr"/>
@@ -2929,11 +2957,11 @@
         </is>
       </c>
       <c r="AZ19" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA19" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/argentina-on-the-go</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/argentina-on-the-go | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB19" t="inlineStr">
@@ -3126,7 +3154,11 @@
       <c r="AI21" t="inlineStr"/>
       <c r="AJ21" t="inlineStr"/>
       <c r="AK21" t="inlineStr"/>
-      <c r="AL21" t="inlineStr"/>
+      <c r="AL21" t="inlineStr">
+        <is>
+          <t>http://www.arthotelsecuador.com</t>
+        </is>
+      </c>
       <c r="AM21" t="inlineStr"/>
       <c r="AN21" t="inlineStr"/>
       <c r="AO21" t="inlineStr"/>
@@ -3149,11 +3181,11 @@
         </is>
       </c>
       <c r="AZ21" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA21" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/arthoteles-ecuador-sa</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/arthoteles-ecuador-sa | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB21" t="inlineStr">
@@ -3470,7 +3502,11 @@
       <c r="AI24" t="inlineStr"/>
       <c r="AJ24" t="inlineStr"/>
       <c r="AK24" t="inlineStr"/>
-      <c r="AL24" t="inlineStr"/>
+      <c r="AL24" t="inlineStr">
+        <is>
+          <t>http://www.avancargo.com</t>
+        </is>
+      </c>
       <c r="AM24" t="inlineStr"/>
       <c r="AN24" t="inlineStr"/>
       <c r="AO24" t="inlineStr"/>
@@ -3493,11 +3529,11 @@
         </is>
       </c>
       <c r="AZ24" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA24" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/avancargo</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/avancargo | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB24" t="inlineStr">
@@ -3714,7 +3750,11 @@
       <c r="AI26" t="inlineStr"/>
       <c r="AJ26" t="inlineStr"/>
       <c r="AK26" t="inlineStr"/>
-      <c r="AL26" t="inlineStr"/>
+      <c r="AL26" t="inlineStr">
+        <is>
+          <t>http://www.bancoestado.cl</t>
+        </is>
+      </c>
       <c r="AM26" t="inlineStr"/>
       <c r="AN26" t="inlineStr"/>
       <c r="AO26" t="inlineStr"/>
@@ -3737,11 +3777,11 @@
         </is>
       </c>
       <c r="AZ26" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA26" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/bancoestado-microempresas/</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/bancoestado-microempresas/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB26" t="inlineStr">
@@ -4194,7 +4234,11 @@
       <c r="AI30" t="inlineStr"/>
       <c r="AJ30" t="inlineStr"/>
       <c r="AK30" t="inlineStr"/>
-      <c r="AL30" t="inlineStr"/>
+      <c r="AL30" t="inlineStr">
+        <is>
+          <t>http://www.bhconsulting.com.ar</t>
+        </is>
+      </c>
       <c r="AM30" t="inlineStr"/>
       <c r="AN30" t="inlineStr"/>
       <c r="AO30" t="inlineStr"/>
@@ -4217,11 +4261,11 @@
         </is>
       </c>
       <c r="AZ30" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA30" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net//find-a-b-corp/company/bh-consulting-srl</t>
+          <t>https://www.bcorporation.net//find-a-b-corp/company/bh-consulting-srl | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB30" t="inlineStr">
@@ -4694,7 +4738,11 @@
       <c r="AI34" t="inlineStr"/>
       <c r="AJ34" t="inlineStr"/>
       <c r="AK34" t="inlineStr"/>
-      <c r="AL34" t="inlineStr"/>
+      <c r="AL34" t="inlineStr">
+        <is>
+          <t>http://www.biogreen.com.ar</t>
+        </is>
+      </c>
       <c r="AM34" t="inlineStr"/>
       <c r="AN34" t="inlineStr"/>
       <c r="AO34" t="inlineStr"/>
@@ -4717,9 +4765,13 @@
         </is>
       </c>
       <c r="AZ34" t="n">
-        <v>21</v>
-      </c>
-      <c r="BA34" t="inlineStr"/>
+        <v>29</v>
+      </c>
+      <c r="BA34" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB34" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -5198,7 +5250,11 @@
       <c r="AI38" t="inlineStr"/>
       <c r="AJ38" t="inlineStr"/>
       <c r="AK38" t="inlineStr"/>
-      <c r="AL38" t="inlineStr"/>
+      <c r="AL38" t="inlineStr">
+        <is>
+          <t>http://www.bligraf.com</t>
+        </is>
+      </c>
       <c r="AM38" t="inlineStr"/>
       <c r="AN38" t="inlineStr"/>
       <c r="AO38" t="inlineStr"/>
@@ -5221,11 +5277,11 @@
         </is>
       </c>
       <c r="AZ38" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="BA38" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/bligraf-sa/</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/bligraf-sa/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB38" t="inlineStr">
@@ -5292,7 +5348,11 @@
       <c r="AI39" t="inlineStr"/>
       <c r="AJ39" t="inlineStr"/>
       <c r="AK39" t="inlineStr"/>
-      <c r="AL39" t="inlineStr"/>
+      <c r="AL39" t="inlineStr">
+        <is>
+          <t>http://www.bolsalea.com</t>
+        </is>
+      </c>
       <c r="AM39" t="inlineStr"/>
       <c r="AN39" t="inlineStr"/>
       <c r="AO39" t="inlineStr"/>
@@ -5315,11 +5375,11 @@
         </is>
       </c>
       <c r="AZ39" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="BA39" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net//find-a-b-corp/company/bolsalea-embalaje-etico-y-sostenible-sl</t>
+          <t>https://www.bcorporation.net//find-a-b-corp/company/bolsalea-embalaje-etico-y-sostenible-sl | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB39" t="inlineStr">
@@ -5660,7 +5720,11 @@
       <c r="AI42" t="inlineStr"/>
       <c r="AJ42" t="inlineStr"/>
       <c r="AK42" t="inlineStr"/>
-      <c r="AL42" t="inlineStr"/>
+      <c r="AL42" t="inlineStr">
+        <is>
+          <t>http://www.bureo.co</t>
+        </is>
+      </c>
       <c r="AM42" t="inlineStr"/>
       <c r="AN42" t="inlineStr"/>
       <c r="AO42" t="inlineStr"/>
@@ -5683,11 +5747,11 @@
         </is>
       </c>
       <c r="AZ42" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA42" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/bureo-inc</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/bureo-inc | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB42" t="inlineStr">
@@ -6004,7 +6068,11 @@
       <c r="AI45" t="inlineStr"/>
       <c r="AJ45" t="inlineStr"/>
       <c r="AK45" t="inlineStr"/>
-      <c r="AL45" t="inlineStr"/>
+      <c r="AL45" t="inlineStr">
+        <is>
+          <t>http://www.campusb.org</t>
+        </is>
+      </c>
       <c r="AM45" t="inlineStr"/>
       <c r="AN45" t="inlineStr"/>
       <c r="AO45" t="inlineStr"/>
@@ -6023,9 +6091,13 @@
         </is>
       </c>
       <c r="AZ45" t="n">
-        <v>29</v>
-      </c>
-      <c r="BA45" t="inlineStr"/>
+        <v>36</v>
+      </c>
+      <c r="BA45" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB45" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -6344,7 +6416,11 @@
       <c r="AI48" t="inlineStr"/>
       <c r="AJ48" t="inlineStr"/>
       <c r="AK48" t="inlineStr"/>
-      <c r="AL48" t="inlineStr"/>
+      <c r="AL48" t="inlineStr">
+        <is>
+          <t>http://www.carryt.co</t>
+        </is>
+      </c>
       <c r="AM48" t="inlineStr"/>
       <c r="AN48" t="inlineStr"/>
       <c r="AO48" t="inlineStr"/>
@@ -6367,11 +6443,11 @@
         </is>
       </c>
       <c r="AZ48" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA48" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/carryt</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/carryt | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB48" t="inlineStr">
@@ -6814,7 +6890,11 @@
       <c r="AI52" t="inlineStr"/>
       <c r="AJ52" t="inlineStr"/>
       <c r="AK52" t="inlineStr"/>
-      <c r="AL52" t="inlineStr"/>
+      <c r="AL52" t="inlineStr">
+        <is>
+          <t>http://www.cebra.com</t>
+        </is>
+      </c>
       <c r="AM52" t="inlineStr"/>
       <c r="AN52" t="inlineStr"/>
       <c r="AO52" t="inlineStr"/>
@@ -6837,11 +6917,11 @@
         </is>
       </c>
       <c r="AZ52" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA52" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/cebra | https://www.bcorporation.net/en-us/find-a-b-corp/company/cebra/</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/cebra | https://www.bcorporation.net/en-us/find-a-b-corp/company/cebra/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB52" t="inlineStr">
@@ -7050,7 +7130,11 @@
       <c r="AI54" t="inlineStr"/>
       <c r="AJ54" t="inlineStr"/>
       <c r="AK54" t="inlineStr"/>
-      <c r="AL54" t="inlineStr"/>
+      <c r="AL54" t="inlineStr">
+        <is>
+          <t>http://www.copayapuconsultores.cl</t>
+        </is>
+      </c>
       <c r="AM54" t="inlineStr"/>
       <c r="AN54" t="inlineStr"/>
       <c r="AO54" t="inlineStr"/>
@@ -7073,11 +7157,11 @@
         </is>
       </c>
       <c r="AZ54" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="BA54" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/centro-de-innovacin-y-emprendimiento-copayapu-consultores-ltda | https://www.bcorporation.net/en-us/find-a-b-corp/company/centro-de-innovacin-y-emprendimiento-copayapu-consultores-ltda/</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/centro-de-innovacin-y-emprendimiento-copayapu-consultores-ltda | https://www.bcorporation.net/en-us/find-a-b-corp/company/centro-de-innovacin-y-emprendimiento-copayapu-consultores-ltda/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB54" t="inlineStr">
@@ -7442,7 +7526,11 @@
       <c r="AI57" t="inlineStr"/>
       <c r="AJ57" t="inlineStr"/>
       <c r="AK57" t="inlineStr"/>
-      <c r="AL57" t="inlineStr"/>
+      <c r="AL57" t="inlineStr">
+        <is>
+          <t>http://www.coda.cl</t>
+        </is>
+      </c>
       <c r="AM57" t="inlineStr"/>
       <c r="AN57" t="inlineStr"/>
       <c r="AO57" t="inlineStr"/>
@@ -7469,11 +7557,11 @@
         </is>
       </c>
       <c r="AZ57" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA57" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/coda</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/coda | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB57" t="inlineStr">
@@ -7562,7 +7650,11 @@
       <c r="AI58" t="inlineStr"/>
       <c r="AJ58" t="inlineStr"/>
       <c r="AK58" t="inlineStr"/>
-      <c r="AL58" t="inlineStr"/>
+      <c r="AL58" t="inlineStr">
+        <is>
+          <t>http://www.ciclofauna.cl</t>
+        </is>
+      </c>
       <c r="AM58" t="inlineStr"/>
       <c r="AN58" t="inlineStr"/>
       <c r="AO58" t="inlineStr"/>
@@ -7585,11 +7677,11 @@
         </is>
       </c>
       <c r="AZ58" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA58" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/ciclo-fauna/</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/ciclo-fauna/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB58" t="inlineStr">
@@ -7678,7 +7770,11 @@
       <c r="AI59" t="inlineStr"/>
       <c r="AJ59" t="inlineStr"/>
       <c r="AK59" t="inlineStr"/>
-      <c r="AL59" t="inlineStr"/>
+      <c r="AL59" t="inlineStr">
+        <is>
+          <t>http://www.comaco.cl</t>
+        </is>
+      </c>
       <c r="AM59" t="inlineStr"/>
       <c r="AN59" t="inlineStr"/>
       <c r="AO59" t="inlineStr"/>
@@ -7701,11 +7797,11 @@
         </is>
       </c>
       <c r="AZ59" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA59" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/comaco | https://www.bcorporation.net/en-us/find-a-b-corp/company/comaco/</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/comaco | https://www.bcorporation.net/en-us/find-a-b-corp/company/comaco/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB59" t="inlineStr">
@@ -7886,7 +7982,11 @@
       <c r="AI61" t="inlineStr"/>
       <c r="AJ61" t="inlineStr"/>
       <c r="AK61" t="inlineStr"/>
-      <c r="AL61" t="inlineStr"/>
+      <c r="AL61" t="inlineStr">
+        <is>
+          <t>http://www.companiadealimentos.com.ar</t>
+        </is>
+      </c>
       <c r="AM61" t="inlineStr"/>
       <c r="AN61" t="inlineStr"/>
       <c r="AO61" t="inlineStr"/>
@@ -7909,11 +8009,11 @@
         </is>
       </c>
       <c r="AZ61" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA61" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/compaia-de-alimentos-y-cereales-sa</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/compaia-de-alimentos-y-cereales-sa | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB61" t="inlineStr">
@@ -8644,7 +8744,11 @@
       <c r="AI67" t="inlineStr"/>
       <c r="AJ67" t="inlineStr"/>
       <c r="AK67" t="inlineStr"/>
-      <c r="AL67" t="inlineStr"/>
+      <c r="AL67" t="inlineStr">
+        <is>
+          <t>http://www.crosshipping.com</t>
+        </is>
+      </c>
       <c r="AM67" t="inlineStr"/>
       <c r="AN67" t="inlineStr"/>
       <c r="AO67" t="inlineStr"/>
@@ -8667,11 +8771,11 @@
         </is>
       </c>
       <c r="AZ67" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA67" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/crosshipping</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/crosshipping | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB67" t="inlineStr">
@@ -10962,7 +11066,11 @@
       <c r="AI86" t="inlineStr"/>
       <c r="AJ86" t="inlineStr"/>
       <c r="AK86" t="inlineStr"/>
-      <c r="AL86" t="inlineStr"/>
+      <c r="AL86" t="inlineStr">
+        <is>
+          <t>http://www.esenciapatagonia.com</t>
+        </is>
+      </c>
       <c r="AM86" t="inlineStr"/>
       <c r="AN86" t="inlineStr"/>
       <c r="AO86" t="inlineStr"/>
@@ -10985,11 +11093,11 @@
         </is>
       </c>
       <c r="AZ86" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="BA86" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/esencia-patagonia | https://www.bcorporation.net/en-us/find-a-b-corp/company/esencia-patagonia/</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/esencia-patagonia | https://www.bcorporation.net/en-us/find-a-b-corp/company/esencia-patagonia/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB86" t="inlineStr">
@@ -11082,7 +11190,11 @@
       <c r="AI87" t="inlineStr"/>
       <c r="AJ87" t="inlineStr"/>
       <c r="AK87" t="inlineStr"/>
-      <c r="AL87" t="inlineStr"/>
+      <c r="AL87" t="inlineStr">
+        <is>
+          <t>http://www.espantapajaros.cl</t>
+        </is>
+      </c>
       <c r="AM87" t="inlineStr"/>
       <c r="AN87" t="inlineStr"/>
       <c r="AO87" t="inlineStr"/>
@@ -11105,11 +11217,11 @@
         </is>
       </c>
       <c r="AZ87" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA87" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net//find-a-b-corp/company/espantapajaros | https://bcorporation.net/directory/espantapajaros</t>
+          <t>https://www.bcorporation.net//find-a-b-corp/company/espantapajaros | https://bcorporation.net/directory/espantapajaros | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB87" t="inlineStr">
@@ -11622,7 +11734,11 @@
       <c r="AI91" t="inlineStr"/>
       <c r="AJ91" t="inlineStr"/>
       <c r="AK91" t="inlineStr"/>
-      <c r="AL91" t="inlineStr"/>
+      <c r="AL91" t="inlineStr">
+        <is>
+          <t>http://www.favima.com</t>
+        </is>
+      </c>
       <c r="AM91" t="inlineStr"/>
       <c r="AN91" t="inlineStr"/>
       <c r="AO91" t="inlineStr"/>
@@ -11645,11 +11761,11 @@
         </is>
       </c>
       <c r="AZ91" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA91" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net//en-us/find-a-b-corp/company/favima</t>
+          <t>https://www.bcorporation.net//en-us/find-a-b-corp/company/favima | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB91" t="inlineStr">
@@ -12134,7 +12250,11 @@
       <c r="AI95" t="inlineStr"/>
       <c r="AJ95" t="inlineStr"/>
       <c r="AK95" t="inlineStr"/>
-      <c r="AL95" t="inlineStr"/>
+      <c r="AL95" t="inlineStr">
+        <is>
+          <t>http://www.freemet.cl</t>
+        </is>
+      </c>
       <c r="AM95" t="inlineStr"/>
       <c r="AN95" t="inlineStr"/>
       <c r="AO95" t="inlineStr"/>
@@ -12157,11 +12277,11 @@
         </is>
       </c>
       <c r="AZ95" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA95" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net//find-a-b-corp/company/freemet-comercial-spa</t>
+          <t>https://www.bcorporation.net//find-a-b-corp/company/freemet-comercial-spa | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB95" t="inlineStr">
@@ -12390,7 +12510,11 @@
       <c r="AI97" t="inlineStr"/>
       <c r="AJ97" t="inlineStr"/>
       <c r="AK97" t="inlineStr"/>
-      <c r="AL97" t="inlineStr"/>
+      <c r="AL97" t="inlineStr">
+        <is>
+          <t>http://www.fruselva.com</t>
+        </is>
+      </c>
       <c r="AM97" t="inlineStr"/>
       <c r="AN97" t="inlineStr"/>
       <c r="AO97" t="inlineStr"/>
@@ -12413,11 +12537,11 @@
         </is>
       </c>
       <c r="AZ97" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA97" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/fruselva-amrica</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/fruselva-amrica | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB97" t="inlineStr">
@@ -13452,7 +13576,11 @@
       <c r="AI106" t="inlineStr"/>
       <c r="AJ106" t="inlineStr"/>
       <c r="AK106" t="inlineStr"/>
-      <c r="AL106" t="inlineStr"/>
+      <c r="AL106" t="inlineStr">
+        <is>
+          <t>http://www.greening-rca.cl</t>
+        </is>
+      </c>
       <c r="AM106" t="inlineStr"/>
       <c r="AN106" t="inlineStr"/>
       <c r="AO106" t="inlineStr"/>
@@ -13475,11 +13603,11 @@
         </is>
       </c>
       <c r="AZ106" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="BA106" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/greening-sp-a | https://www.bcorporation.net/en-us/find-a-b-corp/company/greening-sp-a/</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/greening-sp-a | https://www.bcorporation.net/en-us/find-a-b-corp/company/greening-sp-a/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB106" t="inlineStr">
@@ -14174,7 +14302,11 @@
       <c r="AI112" t="inlineStr"/>
       <c r="AJ112" t="inlineStr"/>
       <c r="AK112" t="inlineStr"/>
-      <c r="AL112" t="inlineStr"/>
+      <c r="AL112" t="inlineStr">
+        <is>
+          <t>http://www.verdical.cl</t>
+        </is>
+      </c>
       <c r="AM112" t="inlineStr"/>
       <c r="AN112" t="inlineStr"/>
       <c r="AO112" t="inlineStr"/>
@@ -14197,11 +14329,11 @@
         </is>
       </c>
       <c r="AZ112" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="BA112" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/grupo-verdical-spa/</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/grupo-verdical-spa/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB112" t="inlineStr">
@@ -14532,7 +14664,11 @@
       <c r="AI115" t="inlineStr"/>
       <c r="AJ115" t="inlineStr"/>
       <c r="AK115" t="inlineStr"/>
-      <c r="AL115" t="inlineStr"/>
+      <c r="AL115" t="inlineStr">
+        <is>
+          <t>http://www.imeko.cl</t>
+        </is>
+      </c>
       <c r="AM115" t="inlineStr"/>
       <c r="AN115" t="inlineStr"/>
       <c r="AO115" t="inlineStr"/>
@@ -14555,11 +14691,11 @@
         </is>
       </c>
       <c r="AZ115" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA115" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/imeko-spa</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/imeko-spa | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB115" t="inlineStr">
@@ -14626,7 +14762,11 @@
       <c r="AI116" t="inlineStr"/>
       <c r="AJ116" t="inlineStr"/>
       <c r="AK116" t="inlineStr"/>
-      <c r="AL116" t="inlineStr"/>
+      <c r="AL116" t="inlineStr">
+        <is>
+          <t>http://www.impacto35.com</t>
+        </is>
+      </c>
       <c r="AM116" t="inlineStr"/>
       <c r="AN116" t="inlineStr"/>
       <c r="AO116" t="inlineStr"/>
@@ -14645,11 +14785,11 @@
         </is>
       </c>
       <c r="AZ116" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="BA116" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/impacto-35/</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/impacto-35/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB116" t="inlineStr">
@@ -14738,7 +14878,11 @@
       <c r="AI117" t="inlineStr"/>
       <c r="AJ117" t="inlineStr"/>
       <c r="AK117" t="inlineStr"/>
-      <c r="AL117" t="inlineStr"/>
+      <c r="AL117" t="inlineStr">
+        <is>
+          <t>http://www.implementasur.com</t>
+        </is>
+      </c>
       <c r="AM117" t="inlineStr"/>
       <c r="AN117" t="inlineStr"/>
       <c r="AO117" t="inlineStr"/>
@@ -14761,11 +14905,11 @@
         </is>
       </c>
       <c r="AZ117" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA117" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/implementa-sur</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/implementa-sur | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB117" t="inlineStr">
@@ -14854,7 +14998,11 @@
       <c r="AI118" t="inlineStr"/>
       <c r="AJ118" t="inlineStr"/>
       <c r="AK118" t="inlineStr"/>
-      <c r="AL118" t="inlineStr"/>
+      <c r="AL118" t="inlineStr">
+        <is>
+          <t>http://www.norte-verde.cl</t>
+        </is>
+      </c>
       <c r="AM118" t="inlineStr"/>
       <c r="AN118" t="inlineStr"/>
       <c r="AO118" t="inlineStr"/>
@@ -14877,11 +15025,11 @@
         </is>
       </c>
       <c r="AZ118" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA118" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/inmobiliaria-norte-verde/</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/inmobiliaria-norte-verde/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB118" t="inlineStr">
@@ -15512,7 +15660,11 @@
       <c r="AI123" t="inlineStr"/>
       <c r="AJ123" t="inlineStr"/>
       <c r="AK123" t="inlineStr"/>
-      <c r="AL123" t="inlineStr"/>
+      <c r="AL123" t="inlineStr">
+        <is>
+          <t>http://www.bontontoys.com</t>
+        </is>
+      </c>
       <c r="AM123" t="inlineStr"/>
       <c r="AN123" t="inlineStr"/>
       <c r="AO123" t="inlineStr"/>
@@ -15535,9 +15687,13 @@
         </is>
       </c>
       <c r="AZ123" t="n">
-        <v>14</v>
-      </c>
-      <c r="BA123" t="inlineStr"/>
+        <v>21</v>
+      </c>
+      <c r="BA123" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB123" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -15890,7 +16046,11 @@
       <c r="AI126" t="inlineStr"/>
       <c r="AJ126" t="inlineStr"/>
       <c r="AK126" t="inlineStr"/>
-      <c r="AL126" t="inlineStr"/>
+      <c r="AL126" t="inlineStr">
+        <is>
+          <t>http://www.islanatura.com</t>
+        </is>
+      </c>
       <c r="AM126" t="inlineStr"/>
       <c r="AN126" t="inlineStr"/>
       <c r="AO126" t="inlineStr"/>
@@ -15917,11 +16077,11 @@
         </is>
       </c>
       <c r="AZ126" t="n">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="BA126" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/isla-natura-exportadora-ltda/ | https://cl.linkedin.com/in/britt-lewis-2a651a28</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/isla-natura-exportadora-ltda/ | https://cl.linkedin.com/in/britt-lewis-2a651a28 | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB126" t="inlineStr">
@@ -16994,7 +17154,11 @@
       <c r="AI135" t="inlineStr"/>
       <c r="AJ135" t="inlineStr"/>
       <c r="AK135" t="inlineStr"/>
-      <c r="AL135" t="inlineStr"/>
+      <c r="AL135" t="inlineStr">
+        <is>
+          <t>http://www.late.cl</t>
+        </is>
+      </c>
       <c r="AM135" t="inlineStr"/>
       <c r="AN135" t="inlineStr"/>
       <c r="AO135" t="inlineStr"/>
@@ -17017,11 +17181,11 @@
         </is>
       </c>
       <c r="AZ135" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="BA135" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/late/</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/late/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB135" t="inlineStr">
@@ -17358,7 +17522,11 @@
       <c r="AI138" t="inlineStr"/>
       <c r="AJ138" t="inlineStr"/>
       <c r="AK138" t="inlineStr"/>
-      <c r="AL138" t="inlineStr"/>
+      <c r="AL138" t="inlineStr">
+        <is>
+          <t>http://www.lofservicios.com</t>
+        </is>
+      </c>
       <c r="AM138" t="inlineStr"/>
       <c r="AN138" t="inlineStr"/>
       <c r="AO138" t="inlineStr"/>
@@ -17381,11 +17549,11 @@
         </is>
       </c>
       <c r="AZ138" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="BA138" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/lof-servicios-spa</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/lof-servicios-spa | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB138" t="inlineStr">
@@ -17482,7 +17650,11 @@
       <c r="AI139" t="inlineStr"/>
       <c r="AJ139" t="inlineStr"/>
       <c r="AK139" t="inlineStr"/>
-      <c r="AL139" t="inlineStr"/>
+      <c r="AL139" t="inlineStr">
+        <is>
+          <t>http://www.lonchera.cl</t>
+        </is>
+      </c>
       <c r="AM139" t="inlineStr"/>
       <c r="AN139" t="inlineStr"/>
       <c r="AO139" t="inlineStr"/>
@@ -17505,11 +17677,11 @@
         </is>
       </c>
       <c r="AZ139" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="BA139" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/lonchera-sp-a | https://www.bcorporation.net/en-us/find-a-b-corp/company/lonchera-sp-a/</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/lonchera-sp-a | https://www.bcorporation.net/en-us/find-a-b-corp/company/lonchera-sp-a/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB139" t="inlineStr">
@@ -17590,7 +17762,11 @@
       <c r="AI140" t="inlineStr"/>
       <c r="AJ140" t="inlineStr"/>
       <c r="AK140" t="inlineStr"/>
-      <c r="AL140" t="inlineStr"/>
+      <c r="AL140" t="inlineStr">
+        <is>
+          <t>http://www.lalucha.com.pe</t>
+        </is>
+      </c>
       <c r="AM140" t="inlineStr"/>
       <c r="AN140" t="inlineStr"/>
       <c r="AO140" t="inlineStr"/>
@@ -17613,9 +17789,13 @@
         </is>
       </c>
       <c r="AZ140" t="n">
-        <v>29</v>
-      </c>
-      <c r="BA140" t="inlineStr"/>
+        <v>36</v>
+      </c>
+      <c r="BA140" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB140" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -17702,7 +17882,11 @@
       <c r="AI141" t="inlineStr"/>
       <c r="AJ141" t="inlineStr"/>
       <c r="AK141" t="inlineStr"/>
-      <c r="AL141" t="inlineStr"/>
+      <c r="AL141" t="inlineStr">
+        <is>
+          <t>http://www.lukkap.cl</t>
+        </is>
+      </c>
       <c r="AM141" t="inlineStr"/>
       <c r="AN141" t="inlineStr"/>
       <c r="AO141" t="inlineStr"/>
@@ -17725,11 +17909,11 @@
         </is>
       </c>
       <c r="AZ141" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA141" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/lukkap-chile</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/lukkap-chile | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB141" t="inlineStr">
@@ -17926,7 +18110,11 @@
       <c r="AI143" t="inlineStr"/>
       <c r="AJ143" t="inlineStr"/>
       <c r="AK143" t="inlineStr"/>
-      <c r="AL143" t="inlineStr"/>
+      <c r="AL143" t="inlineStr">
+        <is>
+          <t>http://www.mpf.com.pe</t>
+        </is>
+      </c>
       <c r="AM143" t="inlineStr"/>
       <c r="AN143" t="inlineStr"/>
       <c r="AO143" t="inlineStr"/>
@@ -17949,11 +18137,11 @@
         </is>
       </c>
       <c r="AZ143" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA143" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/machu-picchu-foods-sac</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/machu-picchu-foods-sac | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB143" t="inlineStr">
@@ -18178,7 +18366,11 @@
       <c r="AI145" t="inlineStr"/>
       <c r="AJ145" t="inlineStr"/>
       <c r="AK145" t="inlineStr"/>
-      <c r="AL145" t="inlineStr"/>
+      <c r="AL145" t="inlineStr">
+        <is>
+          <t>http://www.emarketpeople.com</t>
+        </is>
+      </c>
       <c r="AM145" t="inlineStr"/>
       <c r="AN145" t="inlineStr"/>
       <c r="AO145" t="inlineStr"/>
@@ -18201,11 +18393,11 @@
         </is>
       </c>
       <c r="AZ145" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA145" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/market-people-indumentarias-sp-a/</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/market-people-indumentarias-sp-a/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB145" t="inlineStr">
@@ -18280,7 +18472,11 @@
       <c r="AI146" t="inlineStr"/>
       <c r="AJ146" t="inlineStr"/>
       <c r="AK146" t="inlineStr"/>
-      <c r="AL146" t="inlineStr"/>
+      <c r="AL146" t="inlineStr">
+        <is>
+          <t>http://www.marketgreen.cl</t>
+        </is>
+      </c>
       <c r="AM146" t="inlineStr"/>
       <c r="AN146" t="inlineStr"/>
       <c r="AO146" t="inlineStr"/>
@@ -18303,11 +18499,11 @@
         </is>
       </c>
       <c r="AZ146" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="BA146" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/marketgreen</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/marketgreen | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB146" t="inlineStr">
@@ -18508,7 +18704,11 @@
       <c r="AI148" t="inlineStr"/>
       <c r="AJ148" t="inlineStr"/>
       <c r="AK148" t="inlineStr"/>
-      <c r="AL148" t="inlineStr"/>
+      <c r="AL148" t="inlineStr">
+        <is>
+          <t>http://www.mejores-practicas.com</t>
+        </is>
+      </c>
       <c r="AM148" t="inlineStr"/>
       <c r="AN148" t="inlineStr"/>
       <c r="AO148" t="inlineStr"/>
@@ -18531,11 +18731,11 @@
         </is>
       </c>
       <c r="AZ148" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA148" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/mejores-prcticas | https://www.bcorporation.net/find-a-b-corp/company/mejores-prcticas</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/mejores-prcticas | https://www.bcorporation.net/find-a-b-corp/company/mejores-prcticas | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB148" t="inlineStr">
@@ -18614,7 +18814,11 @@
       <c r="AI149" t="inlineStr"/>
       <c r="AJ149" t="inlineStr"/>
       <c r="AK149" t="inlineStr"/>
-      <c r="AL149" t="inlineStr"/>
+      <c r="AL149" t="inlineStr">
+        <is>
+          <t>http://www.mercadocircular.com</t>
+        </is>
+      </c>
       <c r="AM149" t="inlineStr"/>
       <c r="AN149" t="inlineStr"/>
       <c r="AO149" t="inlineStr"/>
@@ -18637,11 +18841,11 @@
         </is>
       </c>
       <c r="AZ149" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="BA149" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/mercado-circular-sp-a</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/mercado-circular-sp-a | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB149" t="inlineStr">
@@ -18846,7 +19050,11 @@
       <c r="AI151" t="inlineStr"/>
       <c r="AJ151" t="inlineStr"/>
       <c r="AK151" t="inlineStr"/>
-      <c r="AL151" t="inlineStr"/>
+      <c r="AL151" t="inlineStr">
+        <is>
+          <t>http://www.monteswines.com</t>
+        </is>
+      </c>
       <c r="AM151" t="inlineStr"/>
       <c r="AN151" t="inlineStr"/>
       <c r="AO151" t="inlineStr"/>
@@ -18869,11 +19077,11 @@
         </is>
       </c>
       <c r="AZ151" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="BA151" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/montes-wines | https://wineindustryadvisor.com/2024/08/19/montes-wines-earns-prestigious-b-corp-certification/ | https://www.bcorporation.net/en-us/find-a-b-corp/company/montes-wines/</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/montes-wines | https://wineindustryadvisor.com/2024/08/19/montes-wines-earns-prestigious-b-corp-certification/ | https://www.bcorporation.net/en-us/find-a-b-corp/company/montes-wines/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB151" t="inlineStr">
@@ -18950,7 +19158,11 @@
       <c r="AI152" t="inlineStr"/>
       <c r="AJ152" t="inlineStr"/>
       <c r="AK152" t="inlineStr"/>
-      <c r="AL152" t="inlineStr"/>
+      <c r="AL152" t="inlineStr">
+        <is>
+          <t>http://www.natura.com.br</t>
+        </is>
+      </c>
       <c r="AM152" t="inlineStr"/>
       <c r="AN152" t="inlineStr"/>
       <c r="AO152" t="inlineStr"/>
@@ -18973,11 +19185,11 @@
         </is>
       </c>
       <c r="AZ152" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA152" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net//find-a-b-corp/company/natura-cosmeticos-sa</t>
+          <t>https://www.bcorporation.net//find-a-b-corp/company/natura-cosmeticos-sa | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB152" t="inlineStr">
@@ -19048,7 +19260,11 @@
       <c r="AI153" t="inlineStr"/>
       <c r="AJ153" t="inlineStr"/>
       <c r="AK153" t="inlineStr"/>
-      <c r="AL153" t="inlineStr"/>
+      <c r="AL153" t="inlineStr">
+        <is>
+          <t>http://www.neoconsulting.ai</t>
+        </is>
+      </c>
       <c r="AM153" t="inlineStr"/>
       <c r="AN153" t="inlineStr"/>
       <c r="AO153" t="inlineStr"/>
@@ -19071,11 +19287,11 @@
         </is>
       </c>
       <c r="AZ153" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="BA153" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/neo-consulting | https://www.bcorporation.net/en-us/find-a-b-corp/company/neo-consulting/</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/neo-consulting | https://www.bcorporation.net/en-us/find-a-b-corp/company/neo-consulting/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB153" t="inlineStr">
@@ -19164,7 +19380,11 @@
       <c r="AI154" t="inlineStr"/>
       <c r="AJ154" t="inlineStr"/>
       <c r="AK154" t="inlineStr"/>
-      <c r="AL154" t="inlineStr"/>
+      <c r="AL154" t="inlineStr">
+        <is>
+          <t>http://www.newencosmetica.com</t>
+        </is>
+      </c>
       <c r="AM154" t="inlineStr"/>
       <c r="AN154" t="inlineStr"/>
       <c r="AO154" t="inlineStr"/>
@@ -19187,9 +19407,13 @@
         </is>
       </c>
       <c r="AZ154" t="n">
-        <v>21</v>
-      </c>
-      <c r="BA154" t="inlineStr"/>
+        <v>29</v>
+      </c>
+      <c r="BA154" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB154" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -19276,7 +19500,11 @@
       <c r="AI155" t="inlineStr"/>
       <c r="AJ155" t="inlineStr"/>
       <c r="AK155" t="inlineStr"/>
-      <c r="AL155" t="inlineStr"/>
+      <c r="AL155" t="inlineStr">
+        <is>
+          <t>http://www.nodochile.cl</t>
+        </is>
+      </c>
       <c r="AM155" t="inlineStr"/>
       <c r="AN155" t="inlineStr"/>
       <c r="AO155" t="inlineStr"/>
@@ -19299,11 +19527,11 @@
         </is>
       </c>
       <c r="AZ155" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA155" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/nodo-chile</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/nodo-chile | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB155" t="inlineStr">
@@ -19396,7 +19624,11 @@
       <c r="AI156" t="inlineStr"/>
       <c r="AJ156" t="inlineStr"/>
       <c r="AK156" t="inlineStr"/>
-      <c r="AL156" t="inlineStr"/>
+      <c r="AL156" t="inlineStr">
+        <is>
+          <t>http://www.novofarma.com</t>
+        </is>
+      </c>
       <c r="AM156" t="inlineStr"/>
       <c r="AN156" t="inlineStr"/>
       <c r="AO156" t="inlineStr"/>
@@ -19419,11 +19651,11 @@
         </is>
       </c>
       <c r="AZ156" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA156" t="inlineStr">
         <is>
-          <t>https://intuitionlabs.ai/companies/cro/novofarma-service-s-a</t>
+          <t>https://intuitionlabs.ai/companies/cro/novofarma-service-s-a | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB156" t="inlineStr">
@@ -19510,7 +19742,11 @@
       <c r="AI157" t="inlineStr"/>
       <c r="AJ157" t="inlineStr"/>
       <c r="AK157" t="inlineStr"/>
-      <c r="AL157" t="inlineStr"/>
+      <c r="AL157" t="inlineStr">
+        <is>
+          <t>http://www.hotelawa.cl</t>
+        </is>
+      </c>
       <c r="AM157" t="inlineStr"/>
       <c r="AN157" t="inlineStr"/>
       <c r="AO157" t="inlineStr"/>
@@ -19533,11 +19769,11 @@
         </is>
       </c>
       <c r="AZ157" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="BA157" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/hotel-awa</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/hotel-awa | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB157" t="inlineStr">
@@ -19728,7 +19964,11 @@
       <c r="AI159" t="inlineStr"/>
       <c r="AJ159" t="inlineStr"/>
       <c r="AK159" t="inlineStr"/>
-      <c r="AL159" t="inlineStr"/>
+      <c r="AL159" t="inlineStr">
+        <is>
+          <t>http://www.orion.global</t>
+        </is>
+      </c>
       <c r="AM159" t="inlineStr"/>
       <c r="AN159" t="inlineStr"/>
       <c r="AO159" t="inlineStr"/>
@@ -19751,11 +19991,11 @@
         </is>
       </c>
       <c r="AZ159" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA159" t="inlineStr">
         <is>
-          <t>https://g5noticias.cl/2026/01/02/orion-se-convierte-en-la-primera-compania-de-servicios-tecnologicos-en-latinoamerica-en-certificarse-como-empresa-b/</t>
+          <t>https://g5noticias.cl/2026/01/02/orion-se-convierte-en-la-primera-compania-de-servicios-tecnologicos-en-latinoamerica-en-certificarse-como-empresa-b/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB159" t="inlineStr">
@@ -19830,7 +20070,11 @@
       <c r="AI160" t="inlineStr"/>
       <c r="AJ160" t="inlineStr"/>
       <c r="AK160" t="inlineStr"/>
-      <c r="AL160" t="inlineStr"/>
+      <c r="AL160" t="inlineStr">
+        <is>
+          <t>http://www.oyikiltravel.com</t>
+        </is>
+      </c>
       <c r="AM160" t="inlineStr"/>
       <c r="AN160" t="inlineStr"/>
       <c r="AO160" t="inlineStr"/>
@@ -19853,11 +20097,11 @@
         </is>
       </c>
       <c r="AZ160" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="BA160" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/oyikil-sa</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/oyikil-sa | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB160" t="inlineStr">
@@ -19938,7 +20182,11 @@
       <c r="AI161" t="inlineStr"/>
       <c r="AJ161" t="inlineStr"/>
       <c r="AK161" t="inlineStr"/>
-      <c r="AL161" t="inlineStr"/>
+      <c r="AL161" t="inlineStr">
+        <is>
+          <t>http://www.paniwe.cl</t>
+        </is>
+      </c>
       <c r="AM161" t="inlineStr"/>
       <c r="AN161" t="inlineStr"/>
       <c r="AO161" t="inlineStr"/>
@@ -19961,11 +20209,11 @@
         </is>
       </c>
       <c r="AZ161" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="BA161" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/gestin-ambiental-paiwe-limitada</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/gestin-ambiental-paiwe-limitada | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB161" t="inlineStr">
@@ -20054,7 +20302,11 @@
       <c r="AI162" t="inlineStr"/>
       <c r="AJ162" t="inlineStr"/>
       <c r="AK162" t="inlineStr"/>
-      <c r="AL162" t="inlineStr"/>
+      <c r="AL162" t="inlineStr">
+        <is>
+          <t>http://www.pasdenom.cl</t>
+        </is>
+      </c>
       <c r="AM162" t="inlineStr"/>
       <c r="AN162" t="inlineStr"/>
       <c r="AO162" t="inlineStr"/>
@@ -20077,9 +20329,13 @@
         </is>
       </c>
       <c r="AZ162" t="n">
-        <v>21</v>
-      </c>
-      <c r="BA162" t="inlineStr"/>
+        <v>29</v>
+      </c>
+      <c r="BA162" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB162" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -20290,7 +20546,11 @@
       <c r="AI164" t="inlineStr"/>
       <c r="AJ164" t="inlineStr"/>
       <c r="AK164" t="inlineStr"/>
-      <c r="AL164" t="inlineStr"/>
+      <c r="AL164" t="inlineStr">
+        <is>
+          <t>http://www.patagonia-road.com</t>
+        </is>
+      </c>
       <c r="AM164" t="inlineStr"/>
       <c r="AN164" t="inlineStr"/>
       <c r="AO164" t="inlineStr"/>
@@ -20313,11 +20573,11 @@
         </is>
       </c>
       <c r="AZ164" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="BA164" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/patagonia-road</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/patagonia-road | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB164" t="inlineStr">
@@ -20406,7 +20666,11 @@
       <c r="AI165" t="inlineStr"/>
       <c r="AJ165" t="inlineStr"/>
       <c r="AK165" t="inlineStr"/>
-      <c r="AL165" t="inlineStr"/>
+      <c r="AL165" t="inlineStr">
+        <is>
+          <t>http://www.patagua.cl</t>
+        </is>
+      </c>
       <c r="AM165" t="inlineStr"/>
       <c r="AN165" t="inlineStr"/>
       <c r="AO165" t="inlineStr"/>
@@ -20429,9 +20693,13 @@
         </is>
       </c>
       <c r="AZ165" t="n">
-        <v>21</v>
-      </c>
-      <c r="BA165" t="inlineStr"/>
+        <v>29</v>
+      </c>
+      <c r="BA165" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB165" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -20514,7 +20782,11 @@
       <c r="AI166" t="inlineStr"/>
       <c r="AJ166" t="inlineStr"/>
       <c r="AK166" t="inlineStr"/>
-      <c r="AL166" t="inlineStr"/>
+      <c r="AL166" t="inlineStr">
+        <is>
+          <t>http://www.pchconsultora.com</t>
+        </is>
+      </c>
       <c r="AM166" t="inlineStr"/>
       <c r="AN166" t="inlineStr"/>
       <c r="AO166" t="inlineStr"/>
@@ -20537,11 +20809,11 @@
         </is>
       </c>
       <c r="AZ166" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA166" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/pch-consultora</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/pch-consultora | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB166" t="inlineStr">
@@ -20630,7 +20902,11 @@
       <c r="AI167" t="inlineStr"/>
       <c r="AJ167" t="inlineStr"/>
       <c r="AK167" t="inlineStr"/>
-      <c r="AL167" t="inlineStr"/>
+      <c r="AL167" t="inlineStr">
+        <is>
+          <t>http://www.peraltabogados.cl</t>
+        </is>
+      </c>
       <c r="AM167" t="inlineStr"/>
       <c r="AN167" t="inlineStr"/>
       <c r="AO167" t="inlineStr"/>
@@ -20653,11 +20929,11 @@
         </is>
       </c>
       <c r="AZ167" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA167" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/peralta-abogados</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/peralta-abogados | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB167" t="inlineStr">
@@ -20878,7 +21154,11 @@
       <c r="AI169" t="inlineStr"/>
       <c r="AJ169" t="inlineStr"/>
       <c r="AK169" t="inlineStr"/>
-      <c r="AL169" t="inlineStr"/>
+      <c r="AL169" t="inlineStr">
+        <is>
+          <t>http://www.probenefit.cl</t>
+        </is>
+      </c>
       <c r="AM169" t="inlineStr"/>
       <c r="AN169" t="inlineStr"/>
       <c r="AO169" t="inlineStr"/>
@@ -20901,9 +21181,13 @@
         </is>
       </c>
       <c r="AZ169" t="n">
-        <v>36</v>
-      </c>
-      <c r="BA169" t="inlineStr"/>
+        <v>43</v>
+      </c>
+      <c r="BA169" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB169" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -20990,7 +21274,11 @@
       <c r="AI170" t="inlineStr"/>
       <c r="AJ170" t="inlineStr"/>
       <c r="AK170" t="inlineStr"/>
-      <c r="AL170" t="inlineStr"/>
+      <c r="AL170" t="inlineStr">
+        <is>
+          <t>http://www.sancamilo.com</t>
+        </is>
+      </c>
       <c r="AM170" t="inlineStr"/>
       <c r="AN170" t="inlineStr"/>
       <c r="AO170" t="inlineStr"/>
@@ -21013,11 +21301,11 @@
         </is>
       </c>
       <c r="AZ170" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA170" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/productos-san-camilo</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/productos-san-camilo | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB170" t="inlineStr">
@@ -21098,7 +21386,11 @@
       <c r="AI171" t="inlineStr"/>
       <c r="AJ171" t="inlineStr"/>
       <c r="AK171" t="inlineStr"/>
-      <c r="AL171" t="inlineStr"/>
+      <c r="AL171" t="inlineStr">
+        <is>
+          <t>http://www.prolearning.cl</t>
+        </is>
+      </c>
       <c r="AM171" t="inlineStr"/>
       <c r="AN171" t="inlineStr"/>
       <c r="AO171" t="inlineStr"/>
@@ -21121,11 +21413,11 @@
         </is>
       </c>
       <c r="AZ171" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA171" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/prolearning-gestiones-inostroza-pombett-sp-a</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/prolearning-gestiones-inostroza-pombett-sp-a | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB171" t="inlineStr">
@@ -21198,7 +21490,11 @@
       <c r="AI172" t="inlineStr"/>
       <c r="AJ172" t="inlineStr"/>
       <c r="AK172" t="inlineStr"/>
-      <c r="AL172" t="inlineStr"/>
+      <c r="AL172" t="inlineStr">
+        <is>
+          <t>http://www.proximaservicios.cl</t>
+        </is>
+      </c>
       <c r="AM172" t="inlineStr"/>
       <c r="AN172" t="inlineStr"/>
       <c r="AO172" t="inlineStr"/>
@@ -21221,9 +21517,13 @@
         </is>
       </c>
       <c r="AZ172" t="n">
-        <v>7</v>
-      </c>
-      <c r="BA172" t="inlineStr"/>
+        <v>14</v>
+      </c>
+      <c r="BA172" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB172" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -21314,7 +21614,11 @@
       <c r="AI173" t="inlineStr"/>
       <c r="AJ173" t="inlineStr"/>
       <c r="AK173" t="inlineStr"/>
-      <c r="AL173" t="inlineStr"/>
+      <c r="AL173" t="inlineStr">
+        <is>
+          <t>http://www.proyectaimpacto.com</t>
+        </is>
+      </c>
       <c r="AM173" t="inlineStr"/>
       <c r="AN173" t="inlineStr"/>
       <c r="AO173" t="inlineStr"/>
@@ -21337,11 +21641,11 @@
         </is>
       </c>
       <c r="AZ173" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA173" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/proyecta | https://www.bcorporation.net/find-a-b-corp/company/proyecta | https://www.bcorporation.net/en-us/find-a-b-corp/company/proyecta/</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/proyecta | https://www.bcorporation.net/find-a-b-corp/company/proyecta | https://www.bcorporation.net/en-us/find-a-b-corp/company/proyecta/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB173" t="inlineStr">
@@ -21958,7 +22262,11 @@
       <c r="AI179" t="inlineStr"/>
       <c r="AJ179" t="inlineStr"/>
       <c r="AK179" t="inlineStr"/>
-      <c r="AL179" t="inlineStr"/>
+      <c r="AL179" t="inlineStr">
+        <is>
+          <t>http://www.rebeccaadventuretravel.com</t>
+        </is>
+      </c>
       <c r="AM179" t="inlineStr"/>
       <c r="AN179" t="inlineStr"/>
       <c r="AO179" t="inlineStr"/>
@@ -21981,11 +22289,11 @@
         </is>
       </c>
       <c r="AZ179" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA179" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/rebatravel-sa</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/rebatravel-sa | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB179" t="inlineStr">
@@ -22074,7 +22382,11 @@
       <c r="AI180" t="inlineStr"/>
       <c r="AJ180" t="inlineStr"/>
       <c r="AK180" t="inlineStr"/>
-      <c r="AL180" t="inlineStr"/>
+      <c r="AL180" t="inlineStr">
+        <is>
+          <t>http://www.recylink.com</t>
+        </is>
+      </c>
       <c r="AM180" t="inlineStr"/>
       <c r="AN180" t="inlineStr"/>
       <c r="AO180" t="inlineStr"/>
@@ -22097,11 +22409,11 @@
         </is>
       </c>
       <c r="AZ180" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA180" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/recylink</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/recylink | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB180" t="inlineStr">
@@ -22206,7 +22518,11 @@
       <c r="AI181" t="inlineStr"/>
       <c r="AJ181" t="inlineStr"/>
       <c r="AK181" t="inlineStr"/>
-      <c r="AL181" t="inlineStr"/>
+      <c r="AL181" t="inlineStr">
+        <is>
+          <t>http://www.regeneraorganico.cl</t>
+        </is>
+      </c>
       <c r="AM181" t="inlineStr"/>
       <c r="AN181" t="inlineStr"/>
       <c r="AO181" t="inlineStr"/>
@@ -22229,11 +22545,11 @@
         </is>
       </c>
       <c r="AZ181" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA181" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/regenera-orgnico | https://www.bcorporation.net/en-us/find-a-b-corp/company/regenera-orgnico/</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/regenera-orgnico | https://www.bcorporation.net/en-us/find-a-b-corp/company/regenera-orgnico/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB181" t="inlineStr">
@@ -22322,7 +22638,11 @@
       <c r="AI182" t="inlineStr"/>
       <c r="AJ182" t="inlineStr"/>
       <c r="AK182" t="inlineStr"/>
-      <c r="AL182" t="inlineStr"/>
+      <c r="AL182" t="inlineStr">
+        <is>
+          <t>http://www.rheoliglobal.com</t>
+        </is>
+      </c>
       <c r="AM182" t="inlineStr"/>
       <c r="AN182" t="inlineStr"/>
       <c r="AO182" t="inlineStr"/>
@@ -22345,11 +22665,11 @@
         </is>
       </c>
       <c r="AZ182" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA182" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/rheoli-sp-a</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/rheoli-sp-a | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB182" t="inlineStr">
@@ -22438,7 +22758,11 @@
       <c r="AI183" t="inlineStr"/>
       <c r="AJ183" t="inlineStr"/>
       <c r="AK183" t="inlineStr"/>
-      <c r="AL183" t="inlineStr"/>
+      <c r="AL183" t="inlineStr">
+        <is>
+          <t>http://www.risingsun.cl</t>
+        </is>
+      </c>
       <c r="AM183" t="inlineStr"/>
       <c r="AN183" t="inlineStr"/>
       <c r="AO183" t="inlineStr"/>
@@ -22461,9 +22785,13 @@
         </is>
       </c>
       <c r="AZ183" t="n">
-        <v>21</v>
-      </c>
-      <c r="BA183" t="inlineStr"/>
+        <v>29</v>
+      </c>
+      <c r="BA183" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB183" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -22648,7 +22976,11 @@
       <c r="AI185" t="inlineStr"/>
       <c r="AJ185" t="inlineStr"/>
       <c r="AK185" t="inlineStr"/>
-      <c r="AL185" t="inlineStr"/>
+      <c r="AL185" t="inlineStr">
+        <is>
+          <t>http://www.rubtec.cl</t>
+        </is>
+      </c>
       <c r="AM185" t="inlineStr"/>
       <c r="AN185" t="inlineStr"/>
       <c r="AO185" t="inlineStr"/>
@@ -22671,11 +23003,11 @@
         </is>
       </c>
       <c r="AZ185" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="BA185" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/rubtec</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/rubtec | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB185" t="inlineStr">
@@ -22764,7 +23096,11 @@
       <c r="AI186" t="inlineStr"/>
       <c r="AJ186" t="inlineStr"/>
       <c r="AK186" t="inlineStr"/>
-      <c r="AL186" t="inlineStr"/>
+      <c r="AL186" t="inlineStr">
+        <is>
+          <t>http://www.saexpeditions.com</t>
+        </is>
+      </c>
       <c r="AM186" t="inlineStr"/>
       <c r="AN186" t="inlineStr"/>
       <c r="AO186" t="inlineStr"/>
@@ -22787,11 +23123,11 @@
         </is>
       </c>
       <c r="AZ186" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="BA186" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/sa-expeditions</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/sa-expeditions | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB186" t="inlineStr">
@@ -22996,7 +23332,11 @@
       <c r="AI188" t="inlineStr"/>
       <c r="AJ188" t="inlineStr"/>
       <c r="AK188" t="inlineStr"/>
-      <c r="AL188" t="inlineStr"/>
+      <c r="AL188" t="inlineStr">
+        <is>
+          <t>http://www.sembradorcapital.com</t>
+        </is>
+      </c>
       <c r="AM188" t="inlineStr"/>
       <c r="AN188" t="inlineStr"/>
       <c r="AO188" t="inlineStr"/>
@@ -23019,9 +23359,13 @@
         </is>
       </c>
       <c r="AZ188" t="n">
-        <v>21</v>
-      </c>
-      <c r="BA188" t="inlineStr"/>
+        <v>29</v>
+      </c>
+      <c r="BA188" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB188" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -23228,7 +23572,11 @@
       <c r="AI190" t="inlineStr"/>
       <c r="AJ190" t="inlineStr"/>
       <c r="AK190" t="inlineStr"/>
-      <c r="AL190" t="inlineStr"/>
+      <c r="AL190" t="inlineStr">
+        <is>
+          <t>http://www.sofan.cl</t>
+        </is>
+      </c>
       <c r="AM190" t="inlineStr"/>
       <c r="AN190" t="inlineStr"/>
       <c r="AO190" t="inlineStr"/>
@@ -23251,9 +23599,13 @@
         </is>
       </c>
       <c r="AZ190" t="n">
-        <v>29</v>
-      </c>
-      <c r="BA190" t="inlineStr"/>
+        <v>36</v>
+      </c>
+      <c r="BA190" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB190" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -23448,7 +23800,11 @@
       <c r="AI192" t="inlineStr"/>
       <c r="AJ192" t="inlineStr"/>
       <c r="AK192" t="inlineStr"/>
-      <c r="AL192" t="inlineStr"/>
+      <c r="AL192" t="inlineStr">
+        <is>
+          <t>http://www.sigaturismo.com</t>
+        </is>
+      </c>
       <c r="AM192" t="inlineStr"/>
       <c r="AN192" t="inlineStr"/>
       <c r="AO192" t="inlineStr"/>
@@ -23471,11 +23827,11 @@
         </is>
       </c>
       <c r="AZ192" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA192" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/siga-turismo</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/siga-turismo | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB192" t="inlineStr">
@@ -23558,7 +23914,11 @@
       <c r="AI193" t="inlineStr"/>
       <c r="AJ193" t="inlineStr"/>
       <c r="AK193" t="inlineStr"/>
-      <c r="AL193" t="inlineStr"/>
+      <c r="AL193" t="inlineStr">
+        <is>
+          <t>http://www.siigo.com</t>
+        </is>
+      </c>
       <c r="AM193" t="inlineStr"/>
       <c r="AN193" t="inlineStr"/>
       <c r="AO193" t="inlineStr"/>
@@ -23581,9 +23941,13 @@
         </is>
       </c>
       <c r="AZ193" t="n">
-        <v>21</v>
-      </c>
-      <c r="BA193" t="inlineStr"/>
+        <v>29</v>
+      </c>
+      <c r="BA193" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB193" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -23674,7 +24038,11 @@
       <c r="AI194" t="inlineStr"/>
       <c r="AJ194" t="inlineStr"/>
       <c r="AK194" t="inlineStr"/>
-      <c r="AL194" t="inlineStr"/>
+      <c r="AL194" t="inlineStr">
+        <is>
+          <t>http://www.wearesimplicity.com</t>
+        </is>
+      </c>
       <c r="AM194" t="inlineStr"/>
       <c r="AN194" t="inlineStr"/>
       <c r="AO194" t="inlineStr"/>
@@ -23697,11 +24065,11 @@
         </is>
       </c>
       <c r="AZ194" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA194" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/asesorias-simplicity-spa | https://www.bcorporation.net/en-us/find-a-b-corp/company/asesorias-simplicity-spa/</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/asesorias-simplicity-spa | https://www.bcorporation.net/en-us/find-a-b-corp/company/asesorias-simplicity-spa/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB194" t="inlineStr">
@@ -23794,7 +24162,11 @@
       <c r="AI195" t="inlineStr"/>
       <c r="AJ195" t="inlineStr"/>
       <c r="AK195" t="inlineStr"/>
-      <c r="AL195" t="inlineStr"/>
+      <c r="AL195" t="inlineStr">
+        <is>
+          <t>http://www.skinautica.cl</t>
+        </is>
+      </c>
       <c r="AM195" t="inlineStr"/>
       <c r="AN195" t="inlineStr"/>
       <c r="AO195" t="inlineStr"/>
@@ -23817,9 +24189,13 @@
         </is>
       </c>
       <c r="AZ195" t="n">
-        <v>21</v>
-      </c>
-      <c r="BA195" t="inlineStr"/>
+        <v>29</v>
+      </c>
+      <c r="BA195" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB195" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -23918,7 +24294,11 @@
       <c r="AI196" t="inlineStr"/>
       <c r="AJ196" t="inlineStr"/>
       <c r="AK196" t="inlineStr"/>
-      <c r="AL196" t="inlineStr"/>
+      <c r="AL196" t="inlineStr">
+        <is>
+          <t>http://www.socialab.com</t>
+        </is>
+      </c>
       <c r="AM196" t="inlineStr"/>
       <c r="AN196" t="inlineStr"/>
       <c r="AO196" t="inlineStr"/>
@@ -23941,11 +24321,11 @@
         </is>
       </c>
       <c r="AZ196" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA196" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/socialab</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/socialab | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB196" t="inlineStr">
@@ -24148,7 +24528,11 @@
       <c r="AI198" t="inlineStr"/>
       <c r="AJ198" t="inlineStr"/>
       <c r="AK198" t="inlineStr"/>
-      <c r="AL198" t="inlineStr"/>
+      <c r="AL198" t="inlineStr">
+        <is>
+          <t>http://www.southbridgeseguros.cl</t>
+        </is>
+      </c>
       <c r="AM198" t="inlineStr"/>
       <c r="AN198" t="inlineStr"/>
       <c r="AO198" t="inlineStr"/>
@@ -24171,9 +24555,13 @@
         </is>
       </c>
       <c r="AZ198" t="n">
-        <v>21</v>
-      </c>
-      <c r="BA198" t="inlineStr"/>
+        <v>29</v>
+      </c>
+      <c r="BA198" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB198" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -24260,7 +24648,11 @@
       <c r="AI199" t="inlineStr"/>
       <c r="AJ199" t="inlineStr"/>
       <c r="AK199" t="inlineStr"/>
-      <c r="AL199" t="inlineStr"/>
+      <c r="AL199" t="inlineStr">
+        <is>
+          <t>http://www.spheraenergy.com</t>
+        </is>
+      </c>
       <c r="AM199" t="inlineStr"/>
       <c r="AN199" t="inlineStr"/>
       <c r="AO199" t="inlineStr"/>
@@ -24283,11 +24675,11 @@
         </is>
       </c>
       <c r="AZ199" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA199" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/sphera-energy-sp-a</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/sphera-energy-sp-a | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB199" t="inlineStr">
@@ -24492,7 +24884,11 @@
       <c r="AI201" t="inlineStr"/>
       <c r="AJ201" t="inlineStr"/>
       <c r="AK201" t="inlineStr"/>
-      <c r="AL201" t="inlineStr"/>
+      <c r="AL201" t="inlineStr">
+        <is>
+          <t>http://www.symnetics.cl</t>
+        </is>
+      </c>
       <c r="AM201" t="inlineStr"/>
       <c r="AN201" t="inlineStr"/>
       <c r="AO201" t="inlineStr"/>
@@ -24515,11 +24911,11 @@
         </is>
       </c>
       <c r="AZ201" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA201" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/symnetics-chile</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/symnetics-chile | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB201" t="inlineStr">
@@ -24714,7 +25110,11 @@
       <c r="AI203" t="inlineStr"/>
       <c r="AJ203" t="inlineStr"/>
       <c r="AK203" t="inlineStr"/>
-      <c r="AL203" t="inlineStr"/>
+      <c r="AL203" t="inlineStr">
+        <is>
+          <t>http://www.notco.ai</t>
+        </is>
+      </c>
       <c r="AM203" t="inlineStr"/>
       <c r="AN203" t="inlineStr"/>
       <c r="AO203" t="inlineStr"/>
@@ -24737,9 +25137,13 @@
         </is>
       </c>
       <c r="AZ203" t="n">
-        <v>21</v>
-      </c>
-      <c r="BA203" t="inlineStr"/>
+        <v>29</v>
+      </c>
+      <c r="BA203" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB203" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -24830,7 +25234,11 @@
       <c r="AI204" t="inlineStr"/>
       <c r="AJ204" t="inlineStr"/>
       <c r="AK204" t="inlineStr"/>
-      <c r="AL204" t="inlineStr"/>
+      <c r="AL204" t="inlineStr">
+        <is>
+          <t>http://www.thewildfoods.com</t>
+        </is>
+      </c>
       <c r="AM204" t="inlineStr"/>
       <c r="AN204" t="inlineStr"/>
       <c r="AO204" t="inlineStr"/>
@@ -24853,11 +25261,11 @@
         </is>
       </c>
       <c r="AZ204" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA204" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/the-wild-foods</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/the-wild-foods | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB204" t="inlineStr">
@@ -25058,7 +25466,11 @@
       <c r="AI206" t="inlineStr"/>
       <c r="AJ206" t="inlineStr"/>
       <c r="AK206" t="inlineStr"/>
-      <c r="AL206" t="inlineStr"/>
+      <c r="AL206" t="inlineStr">
+        <is>
+          <t>http://www.tironi.cl</t>
+        </is>
+      </c>
       <c r="AM206" t="inlineStr"/>
       <c r="AN206" t="inlineStr"/>
       <c r="AO206" t="inlineStr"/>
@@ -25081,9 +25493,13 @@
         </is>
       </c>
       <c r="AZ206" t="n">
-        <v>21</v>
-      </c>
-      <c r="BA206" t="inlineStr"/>
+        <v>29</v>
+      </c>
+      <c r="BA206" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB206" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -25178,7 +25594,11 @@
       <c r="AI207" t="inlineStr"/>
       <c r="AJ207" t="inlineStr"/>
       <c r="AK207" t="inlineStr"/>
-      <c r="AL207" t="inlineStr"/>
+      <c r="AL207" t="inlineStr">
+        <is>
+          <t>http://www.pegasconsentido.cl</t>
+        </is>
+      </c>
       <c r="AM207" t="inlineStr"/>
       <c r="AN207" t="inlineStr"/>
       <c r="AO207" t="inlineStr"/>
@@ -25201,11 +25621,11 @@
         </is>
       </c>
       <c r="AZ207" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA207" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/pegas-con-sentido | https://www.elmostrador.cl/mercados/2015/09/17/pegas-con-sentido-el-sello-de-la-generacion-y-a-la-hora-de-buscar-trabajo/</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/pegas-con-sentido | https://www.elmostrador.cl/mercados/2015/09/17/pegas-con-sentido-el-sello-de-la-generacion-y-a-la-hora-de-buscar-trabajo/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB207" t="inlineStr">
@@ -25294,7 +25714,11 @@
       <c r="AI208" t="inlineStr"/>
       <c r="AJ208" t="inlineStr"/>
       <c r="AK208" t="inlineStr"/>
-      <c r="AL208" t="inlineStr"/>
+      <c r="AL208" t="inlineStr">
+        <is>
+          <t>http://www.trasiegowines.com</t>
+        </is>
+      </c>
       <c r="AM208" t="inlineStr"/>
       <c r="AN208" t="inlineStr"/>
       <c r="AO208" t="inlineStr"/>
@@ -25317,11 +25741,11 @@
         </is>
       </c>
       <c r="AZ208" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA208" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/trasiego-wines-sa</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/trasiego-wines-sa | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB208" t="inlineStr">
@@ -25408,7 +25832,11 @@
       <c r="AI209" t="inlineStr"/>
       <c r="AJ209" t="inlineStr"/>
       <c r="AK209" t="inlineStr"/>
-      <c r="AL209" t="inlineStr"/>
+      <c r="AL209" t="inlineStr">
+        <is>
+          <t>http://www.trayecta.cl</t>
+        </is>
+      </c>
       <c r="AM209" t="inlineStr"/>
       <c r="AN209" t="inlineStr"/>
       <c r="AO209" t="inlineStr"/>
@@ -25431,9 +25859,13 @@
         </is>
       </c>
       <c r="AZ209" t="n">
-        <v>14</v>
-      </c>
-      <c r="BA209" t="inlineStr"/>
+        <v>21</v>
+      </c>
+      <c r="BA209" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB209" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -25532,7 +25964,11 @@
       <c r="AI210" t="inlineStr"/>
       <c r="AJ210" t="inlineStr"/>
       <c r="AK210" t="inlineStr"/>
-      <c r="AL210" t="inlineStr"/>
+      <c r="AL210" t="inlineStr">
+        <is>
+          <t>http://www.triciclos.cl</t>
+        </is>
+      </c>
       <c r="AM210" t="inlineStr"/>
       <c r="AN210" t="inlineStr"/>
       <c r="AO210" t="inlineStr"/>
@@ -25555,11 +25991,11 @@
         </is>
       </c>
       <c r="AZ210" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA210" t="inlineStr">
         <is>
-          <t>https://chocale.cl/2026/05/chile-lidera-en-empresas-b-en-latinoamerica-ya-hay-cerca-de-270-certificadas/ | https://www.bcorporation.net/find-a-b-corp/company/triciclos-brasil | https://latamlist.com/1-3-of-latin-americas-b-corps-are-registered-in-chile/ | https://www.marcachile.cl/en/diez-empresas-chilenas-que-pusieron-el-reciclaje-en-el-centro-de-su-negocio/</t>
+          <t>https://chocale.cl/2026/05/chile-lidera-en-empresas-b-en-latinoamerica-ya-hay-cerca-de-270-certificadas/ | https://www.bcorporation.net/find-a-b-corp/company/triciclos-brasil | https://latamlist.com/1-3-of-latin-americas-b-corps-are-registered-in-chile/ | https://www.marcachile.cl/en/diez-empresas-chilenas-que-pusieron-el-reciclaje-en-el-centro-de-su-negocio/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB210" t="inlineStr">
@@ -25634,7 +26070,11 @@
       <c r="AI211" t="inlineStr"/>
       <c r="AJ211" t="inlineStr"/>
       <c r="AK211" t="inlineStr"/>
-      <c r="AL211" t="inlineStr"/>
+      <c r="AL211" t="inlineStr">
+        <is>
+          <t>http://www.unibag.cl</t>
+        </is>
+      </c>
       <c r="AM211" t="inlineStr"/>
       <c r="AN211" t="inlineStr"/>
       <c r="AO211" t="inlineStr"/>
@@ -25657,9 +26097,13 @@
         </is>
       </c>
       <c r="AZ211" t="n">
-        <v>7</v>
-      </c>
-      <c r="BA211" t="inlineStr"/>
+        <v>14</v>
+      </c>
+      <c r="BA211" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB211" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -25738,7 +26182,11 @@
       <c r="AI212" t="inlineStr"/>
       <c r="AJ212" t="inlineStr"/>
       <c r="AK212" t="inlineStr"/>
-      <c r="AL212" t="inlineStr"/>
+      <c r="AL212" t="inlineStr">
+        <is>
+          <t>http://www.unplastify.com</t>
+        </is>
+      </c>
       <c r="AM212" t="inlineStr"/>
       <c r="AN212" t="inlineStr"/>
       <c r="AO212" t="inlineStr"/>
@@ -25761,11 +26209,11 @@
         </is>
       </c>
       <c r="AZ212" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA212" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net//en-us/find-a-b-corp/company/unplastify</t>
+          <t>https://www.bcorporation.net//en-us/find-a-b-corp/company/unplastify | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB212" t="inlineStr">
@@ -25854,7 +26302,11 @@
       <c r="AI213" t="inlineStr"/>
       <c r="AJ213" t="inlineStr"/>
       <c r="AK213" t="inlineStr"/>
-      <c r="AL213" t="inlineStr"/>
+      <c r="AL213" t="inlineStr">
+        <is>
+          <t>http://www.urbani.cl</t>
+        </is>
+      </c>
       <c r="AM213" t="inlineStr"/>
       <c r="AN213" t="inlineStr"/>
       <c r="AO213" t="inlineStr"/>
@@ -25877,9 +26329,13 @@
         </is>
       </c>
       <c r="AZ213" t="n">
-        <v>29</v>
-      </c>
-      <c r="BA213" t="inlineStr"/>
+        <v>36</v>
+      </c>
+      <c r="BA213" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB213" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -26104,7 +26560,11 @@
       <c r="AI215" t="inlineStr"/>
       <c r="AJ215" t="inlineStr"/>
       <c r="AK215" t="inlineStr"/>
-      <c r="AL215" t="inlineStr"/>
+      <c r="AL215" t="inlineStr">
+        <is>
+          <t>http://www.xn--vialosvascos-bhb.cl</t>
+        </is>
+      </c>
       <c r="AM215" t="inlineStr"/>
       <c r="AN215" t="inlineStr"/>
       <c r="AO215" t="inlineStr"/>
@@ -26127,11 +26587,11 @@
         </is>
       </c>
       <c r="AZ215" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="BA215" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/los-vascos</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/los-vascos | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB215" t="inlineStr">
@@ -26212,7 +26672,11 @@
       <c r="AI216" t="inlineStr"/>
       <c r="AJ216" t="inlineStr"/>
       <c r="AK216" t="inlineStr"/>
-      <c r="AL216" t="inlineStr"/>
+      <c r="AL216" t="inlineStr">
+        <is>
+          <t>http://www.montgras.cl</t>
+        </is>
+      </c>
       <c r="AM216" t="inlineStr"/>
       <c r="AN216" t="inlineStr"/>
       <c r="AO216" t="inlineStr"/>
@@ -26235,11 +26699,11 @@
         </is>
       </c>
       <c r="AZ216" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="BA216" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/via-mont-gras | https://www.bcorporation.net/en-us/find-a-b-corp/company/via-mont-gras/</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/via-mont-gras | https://www.bcorporation.net/en-us/find-a-b-corp/company/via-mont-gras/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB216" t="inlineStr">
@@ -26328,7 +26792,11 @@
       <c r="AI217" t="inlineStr"/>
       <c r="AJ217" t="inlineStr"/>
       <c r="AK217" t="inlineStr"/>
-      <c r="AL217" t="inlineStr"/>
+      <c r="AL217" t="inlineStr">
+        <is>
+          <t>http://www.polkura.cl</t>
+        </is>
+      </c>
       <c r="AM217" t="inlineStr"/>
       <c r="AN217" t="inlineStr"/>
       <c r="AO217" t="inlineStr"/>
@@ -26351,11 +26819,11 @@
         </is>
       </c>
       <c r="AZ217" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA217" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/vina-polkura-sa</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/vina-polkura-sa | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB217" t="inlineStr">
@@ -26444,7 +26912,11 @@
       <c r="AI218" t="inlineStr"/>
       <c r="AJ218" t="inlineStr"/>
       <c r="AK218" t="inlineStr"/>
-      <c r="AL218" t="inlineStr"/>
+      <c r="AL218" t="inlineStr">
+        <is>
+          <t>http://www.emiliana.cl</t>
+        </is>
+      </c>
       <c r="AM218" t="inlineStr"/>
       <c r="AN218" t="inlineStr"/>
       <c r="AO218" t="inlineStr"/>
@@ -26467,11 +26939,11 @@
         </is>
       </c>
       <c r="AZ218" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA218" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/emiliana-vineyards</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/emiliana-vineyards | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB218" t="inlineStr">
@@ -26572,7 +27044,11 @@
       <c r="AI219" t="inlineStr"/>
       <c r="AJ219" t="inlineStr"/>
       <c r="AK219" t="inlineStr"/>
-      <c r="AL219" t="inlineStr"/>
+      <c r="AL219" t="inlineStr">
+        <is>
+          <t>http://www.virutexilko.com</t>
+        </is>
+      </c>
       <c r="AM219" t="inlineStr"/>
       <c r="AN219" t="inlineStr"/>
       <c r="AO219" t="inlineStr"/>
@@ -26595,9 +27071,13 @@
         </is>
       </c>
       <c r="AZ219" t="n">
-        <v>21</v>
-      </c>
-      <c r="BA219" t="inlineStr"/>
+        <v>29</v>
+      </c>
+      <c r="BA219" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB219" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -26688,7 +27168,11 @@
       <c r="AI220" t="inlineStr"/>
       <c r="AJ220" t="inlineStr"/>
       <c r="AK220" t="inlineStr"/>
-      <c r="AL220" t="inlineStr"/>
+      <c r="AL220" t="inlineStr">
+        <is>
+          <t>http://www.vitafoods.com</t>
+        </is>
+      </c>
       <c r="AM220" t="inlineStr"/>
       <c r="AN220" t="inlineStr"/>
       <c r="AO220" t="inlineStr"/>
@@ -26711,11 +27195,11 @@
         </is>
       </c>
       <c r="AZ220" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="BA220" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/find-a-b-corp/company/vita-foods | https://www.bcorporation.net/en-us/find-a-b-corp/company/vita-foods/</t>
+          <t>https://www.bcorporation.net/find-a-b-corp/company/vita-foods | https://www.bcorporation.net/en-us/find-a-b-corp/company/vita-foods/ | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB220" t="inlineStr">
@@ -26790,7 +27274,11 @@
       <c r="AI221" t="inlineStr"/>
       <c r="AJ221" t="inlineStr"/>
       <c r="AK221" t="inlineStr"/>
-      <c r="AL221" t="inlineStr"/>
+      <c r="AL221" t="inlineStr">
+        <is>
+          <t>http://www.wherex.com</t>
+        </is>
+      </c>
       <c r="AM221" t="inlineStr"/>
       <c r="AN221" t="inlineStr"/>
       <c r="AO221" t="inlineStr"/>
@@ -26813,9 +27301,13 @@
         </is>
       </c>
       <c r="AZ221" t="n">
-        <v>7</v>
-      </c>
-      <c r="BA221" t="inlineStr"/>
+        <v>14</v>
+      </c>
+      <c r="BA221" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB221" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -27038,7 +27530,11 @@
       <c r="AI223" t="inlineStr"/>
       <c r="AJ223" t="inlineStr"/>
       <c r="AK223" t="inlineStr"/>
-      <c r="AL223" t="inlineStr"/>
+      <c r="AL223" t="inlineStr">
+        <is>
+          <t>http://www.wildlama.com</t>
+        </is>
+      </c>
       <c r="AM223" t="inlineStr"/>
       <c r="AN223" t="inlineStr"/>
       <c r="AO223" t="inlineStr"/>
@@ -27061,9 +27557,13 @@
         </is>
       </c>
       <c r="AZ223" t="n">
-        <v>29</v>
-      </c>
-      <c r="BA223" t="inlineStr"/>
+        <v>36</v>
+      </c>
+      <c r="BA223" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/ (búsqueda de organizaciones)</t>
+        </is>
+      </c>
       <c r="BB223" t="inlineStr">
         <is>
           <t>2026-10-20</t>
@@ -27150,7 +27650,11 @@
       <c r="AI224" t="inlineStr"/>
       <c r="AJ224" t="inlineStr"/>
       <c r="AK224" t="inlineStr"/>
-      <c r="AL224" t="inlineStr"/>
+      <c r="AL224" t="inlineStr">
+        <is>
+          <t>http://www.xinerlink.cl</t>
+        </is>
+      </c>
       <c r="AM224" t="inlineStr"/>
       <c r="AN224" t="inlineStr"/>
       <c r="AO224" t="inlineStr"/>
@@ -27173,11 +27677,11 @@
         </is>
       </c>
       <c r="AZ224" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="BA224" t="inlineStr">
         <is>
-          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/xiner-link-sa</t>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/xiner-link-sa | https://www.apollo.io/ (búsqueda de organizaciones)</t>
         </is>
       </c>
       <c r="BB224" t="inlineStr">

</xml_diff>

<commit_message>
Peor rendimiento económico: resultados de 4 revisiones y nivel «En observación»
- Resultados de los 3 lotes (186 empresas con sede en Chile) y del barrido
  temático en data/raw/rendimiento/. Cuando dos revisiones cubren la misma
  empresa se unen sin repetir hechos y se publica la confianza más baja.
- Nuevo nivel «En observación»: ventas o utilidades a la baja sin pérdidas, o
  problemas ya superados. «Negativo» exige pérdidas, cierres, despidos, deuda
  o rescate en los últimos tres años.
- revision_editorial.json registra las decisiones manuales con su motivo,
  que se muestra en la ficha.
- Corrige la vista de alertas: las secciones se mostraban como texto
  «[object HTMLHeadingElement]».
- Traduce 14 nombres de industria de la taxonomía nueva de B Lab que
  seguían en inglés.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H1ZHr5EuMixHqUzfpFW6bc
</commit_message>
<xml_diff>
--- a/data/empresas_b_chile.xlsx
+++ b/data/empresas_b_chile.xlsx
@@ -1036,7 +1036,7 @@
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ4" t="inlineStr"/>
@@ -1203,7 +1203,7 @@
       </c>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ5" t="inlineStr"/>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="AI6" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ6" t="inlineStr"/>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="AI8" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ8" t="inlineStr"/>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="AI9" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ9" t="inlineStr"/>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="AI10" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ10" t="inlineStr"/>
@@ -2065,7 +2065,7 @@
       </c>
       <c r="AI11" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ11" t="inlineStr"/>
@@ -2200,7 +2200,7 @@
       <c r="AH12" t="inlineStr"/>
       <c r="AI12" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ12" t="inlineStr"/>
@@ -2327,7 +2327,7 @@
       <c r="AH13" t="inlineStr"/>
       <c r="AI13" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ13" t="inlineStr"/>
@@ -2440,7 +2440,7 @@
       <c r="AH14" t="inlineStr"/>
       <c r="AI14" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ14" t="inlineStr"/>
@@ -2686,7 +2686,7 @@
       <c r="AH16" t="inlineStr"/>
       <c r="AI16" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ16" t="inlineStr"/>
@@ -2805,7 +2805,7 @@
       <c r="AH17" t="inlineStr"/>
       <c r="AI17" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ17" t="inlineStr"/>
@@ -2944,7 +2944,7 @@
       <c r="AH18" t="inlineStr"/>
       <c r="AI18" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ18" t="inlineStr"/>
@@ -3192,7 +3192,7 @@
       <c r="AH20" t="inlineStr"/>
       <c r="AI20" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ20" t="inlineStr"/>
@@ -3420,7 +3420,7 @@
       <c r="AH22" t="inlineStr"/>
       <c r="AI22" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ22" t="inlineStr"/>
@@ -3547,7 +3547,7 @@
       <c r="AH23" t="inlineStr"/>
       <c r="AI23" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ23" t="inlineStr"/>
@@ -3789,7 +3789,7 @@
       <c r="AH25" t="inlineStr"/>
       <c r="AI25" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ25" t="inlineStr"/>
@@ -3932,7 +3932,7 @@
       <c r="AH26" t="inlineStr"/>
       <c r="AI26" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ26" t="inlineStr"/>
@@ -4065,7 +4065,7 @@
       <c r="AH27" t="inlineStr"/>
       <c r="AI27" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ27" t="inlineStr"/>
@@ -4200,7 +4200,7 @@
       <c r="AH28" t="inlineStr"/>
       <c r="AI28" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ28" t="inlineStr"/>
@@ -4331,11 +4331,19 @@
       <c r="AH29" t="inlineStr"/>
       <c r="AI29" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
-        </is>
-      </c>
-      <c r="AJ29" t="inlineStr"/>
-      <c r="AK29" t="inlineStr"/>
+          <t>Negativo</t>
+        </is>
+      </c>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>Cierre (2025-03): En un plan de reestructuración despidió a unas 30 personas y cerró operaciones en Colombia, Ecuador, Perú, Argentina y Brasil; continúa solo en Chile, México y España. | Despidos (2023-01): Despidió a cerca del 30% de su plantilla en enero de 2023 (tras un recorte de unas 30 personas en agosto de 2022); su CEO lo atribuyó al complejo entorno económico mundial.</t>
+        </is>
+      </c>
+      <c r="AK29" t="inlineStr">
+        <is>
+          <t>La empresa declaró tener más de cinco años de caja y que Chile, México y España generan el 94% de sus ingresos; el repliegue busca concentrarse en el mercado de EE.UU. No se encontraron cifras de pérdidas publicadas ni noticias posteriores a marzo de 2025.</t>
+        </is>
+      </c>
       <c r="AL29" t="inlineStr"/>
       <c r="AM29" t="inlineStr"/>
       <c r="AN29" t="inlineStr"/>
@@ -4575,7 +4583,7 @@
       <c r="AH31" t="inlineStr"/>
       <c r="AI31" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ31" t="inlineStr"/>
@@ -4643,7 +4651,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Professional, scientific and technical services</t>
+          <t>Servicios profesionales, científicos y técnicos</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -4702,7 +4710,7 @@
       <c r="AH32" t="inlineStr"/>
       <c r="AI32" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ32" t="inlineStr"/>
@@ -4857,7 +4865,7 @@
       </c>
       <c r="AI33" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ33" t="inlineStr"/>
@@ -5119,7 +5127,7 @@
       </c>
       <c r="AI35" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ35" t="inlineStr"/>
@@ -5266,7 +5274,7 @@
       </c>
       <c r="AI36" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ36" t="inlineStr"/>
@@ -5401,7 +5409,7 @@
       <c r="AH37" t="inlineStr"/>
       <c r="AI37" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ37" t="inlineStr"/>
@@ -5516,7 +5524,7 @@
       <c r="AH38" t="inlineStr"/>
       <c r="AI38" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ38" t="inlineStr"/>
@@ -5760,7 +5768,7 @@
       <c r="AH40" t="inlineStr"/>
       <c r="AI40" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ40" t="inlineStr"/>
@@ -5891,7 +5899,7 @@
       <c r="AH41" t="inlineStr"/>
       <c r="AI41" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ41" t="inlineStr"/>
@@ -6141,7 +6149,7 @@
       <c r="AH43" t="inlineStr"/>
       <c r="AI43" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ43" t="inlineStr"/>
@@ -6268,7 +6276,7 @@
       <c r="AH44" t="inlineStr"/>
       <c r="AI44" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ44" t="inlineStr"/>
@@ -6506,7 +6514,7 @@
       <c r="AH46" t="inlineStr"/>
       <c r="AI46" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ46" t="inlineStr"/>
@@ -6633,7 +6641,7 @@
       <c r="AH47" t="inlineStr"/>
       <c r="AI47" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ47" t="inlineStr"/>
@@ -6697,7 +6705,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Postal and courier activities</t>
+          <t>Servicios postales y de mensajería</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -6877,7 +6885,7 @@
       <c r="AH49" t="inlineStr"/>
       <c r="AI49" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ49" t="inlineStr"/>
@@ -7000,7 +7008,7 @@
       <c r="AH50" t="inlineStr"/>
       <c r="AI50" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ50" t="inlineStr"/>
@@ -7123,7 +7131,7 @@
       <c r="AH51" t="inlineStr"/>
       <c r="AI51" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ51" t="inlineStr"/>
@@ -7254,7 +7262,7 @@
       <c r="AH52" t="inlineStr"/>
       <c r="AI52" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ52" t="inlineStr"/>
@@ -7322,7 +7330,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Waste treatment and disposal</t>
+          <t>Tratamiento de residuos</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -7508,7 +7516,7 @@
       <c r="AH54" t="inlineStr"/>
       <c r="AI54" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ54" t="inlineStr"/>
@@ -7655,7 +7663,7 @@
       <c r="AH55" t="inlineStr"/>
       <c r="AI55" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ55" t="inlineStr"/>
@@ -7782,7 +7790,7 @@
       <c r="AH56" t="inlineStr"/>
       <c r="AI56" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ56" t="inlineStr"/>
@@ -7925,7 +7933,7 @@
       <c r="AH57" t="inlineStr"/>
       <c r="AI57" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ57" t="inlineStr"/>
@@ -8056,7 +8064,7 @@
       <c r="AH58" t="inlineStr"/>
       <c r="AI58" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ58" t="inlineStr"/>
@@ -8183,7 +8191,7 @@
       <c r="AH59" t="inlineStr"/>
       <c r="AI59" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ59" t="inlineStr"/>
@@ -8302,7 +8310,7 @@
       <c r="AH60" t="inlineStr"/>
       <c r="AI60" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ60" t="inlineStr"/>
@@ -8572,11 +8580,19 @@
       </c>
       <c r="AI62" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
-        </is>
-      </c>
-      <c r="AJ62" t="inlineStr"/>
-      <c r="AK62" t="inlineStr"/>
+          <t>Negativo</t>
+        </is>
+      </c>
+      <c r="AJ62" t="inlineStr">
+        <is>
+          <t>Pérdidas (2025-05): Reportó pérdidas en el primer trimestre de 2025: ingresos -3,15% a $22.709 millones y línea de colchones con pérdida de $1.358 millones (vs. ganancia de $124 millones un año antes). | Despidos (2025-05): Aplicó un ajuste de gastos de fabricación y administración que implicó $1.357 millones en indemnizaciones (primer trimestre de 2025). | Caída de ventas (2025): Las ventas de 2025 cayeron 5,09% respecto del período anterior por la contracción del mercado de bienes durables, afectando a ambos segmentos (especialmente colchones). | Pérdidas (2024): El análisis razonado de diciembre de 2025 muestra como comparativo una pérdida de unos $935 millones en 2024 (cifra en miles de pesos, unidad inferida).</t>
+        </is>
+      </c>
+      <c r="AK62" t="inlineStr">
+        <is>
+          <t>En 2025 volvió a utilidades: el análisis razonado de diciembre de 2025 muestra una ganancia de unos $826 millones frente a la pérdida de unos $935 millones de 2024, con EBITDA de unos $8.915 millones (vs. $4.870 millones), pese a la caída de ventas. En 2025 comenzó a fabricar colchones Sealy bajo licencia. No se encontró reorganización judicial ni liquidación. Unidades monetarias inferidas del propio informe (miles de pesos).</t>
+        </is>
+      </c>
       <c r="AL62" t="inlineStr"/>
       <c r="AM62" t="inlineStr"/>
       <c r="AN62" t="inlineStr"/>
@@ -8834,7 +8850,7 @@
       </c>
       <c r="AI64" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ64" t="inlineStr"/>
@@ -9086,7 +9102,7 @@
       <c r="AH66" t="inlineStr"/>
       <c r="AI66" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ66" t="inlineStr"/>
@@ -9158,7 +9174,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Other transport equipment</t>
+          <t>Otros equipos de transporte</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -9344,7 +9360,7 @@
       <c r="AH68" t="inlineStr"/>
       <c r="AI68" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ68" t="inlineStr"/>
@@ -9473,7 +9489,7 @@
       <c r="AH69" t="inlineStr"/>
       <c r="AI69" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ69" t="inlineStr"/>
@@ -9600,7 +9616,7 @@
       <c r="AH70" t="inlineStr"/>
       <c r="AI70" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ70" t="inlineStr"/>
@@ -9735,7 +9751,7 @@
       <c r="AH71" t="inlineStr"/>
       <c r="AI71" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ71" t="inlineStr"/>
@@ -9858,7 +9874,7 @@
       <c r="AH72" t="inlineStr"/>
       <c r="AI72" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ72" t="inlineStr"/>
@@ -9985,7 +10001,7 @@
       <c r="AH73" t="inlineStr"/>
       <c r="AI73" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ73" t="inlineStr"/>
@@ -10118,7 +10134,7 @@
       <c r="AH74" t="inlineStr"/>
       <c r="AI74" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ74" t="inlineStr"/>
@@ -10245,7 +10261,7 @@
       <c r="AH75" t="inlineStr"/>
       <c r="AI75" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ75" t="inlineStr"/>
@@ -10372,7 +10388,7 @@
       <c r="AH76" t="inlineStr"/>
       <c r="AI76" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ76" t="inlineStr"/>
@@ -10507,7 +10523,7 @@
       <c r="AH77" t="inlineStr"/>
       <c r="AI77" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ77" t="inlineStr"/>
@@ -10642,7 +10658,7 @@
       <c r="AH78" t="inlineStr"/>
       <c r="AI78" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ78" t="inlineStr"/>
@@ -10773,7 +10789,7 @@
       <c r="AH79" t="inlineStr"/>
       <c r="AI79" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ79" t="inlineStr"/>
@@ -10896,7 +10912,7 @@
       <c r="AH80" t="inlineStr"/>
       <c r="AI80" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ80" t="inlineStr"/>
@@ -11031,7 +11047,7 @@
       <c r="AH81" t="inlineStr"/>
       <c r="AI81" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ81" t="inlineStr"/>
@@ -11162,7 +11178,7 @@
       <c r="AH82" t="inlineStr"/>
       <c r="AI82" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ82" t="inlineStr"/>
@@ -11295,7 +11311,7 @@
       <c r="AH83" t="inlineStr"/>
       <c r="AI83" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ83" t="inlineStr"/>
@@ -11418,7 +11434,7 @@
       <c r="AH84" t="inlineStr"/>
       <c r="AI84" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ84" t="inlineStr"/>
@@ -11482,7 +11498,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Professional, scientific and technical services</t>
+          <t>Servicios profesionales, científicos y técnicos</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -11541,7 +11557,7 @@
       <c r="AH85" t="inlineStr"/>
       <c r="AI85" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ85" t="inlineStr"/>
@@ -11736,7 +11752,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Restaurants and food service</t>
+          <t>Restaurantes y servicios de alimentación</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -11799,7 +11815,7 @@
       <c r="AH87" t="inlineStr"/>
       <c r="AI87" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ87" t="inlineStr"/>
@@ -11930,7 +11946,7 @@
       <c r="AH88" t="inlineStr"/>
       <c r="AI88" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ88" t="inlineStr"/>
@@ -12069,7 +12085,7 @@
       </c>
       <c r="AI89" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ89" t="inlineStr"/>
@@ -12216,7 +12232,7 @@
       </c>
       <c r="AI90" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ90" t="inlineStr"/>
@@ -12371,7 +12387,7 @@
       <c r="AH91" t="inlineStr"/>
       <c r="AI91" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ91" t="inlineStr"/>
@@ -12506,7 +12522,7 @@
       </c>
       <c r="AI92" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ92" t="inlineStr"/>
@@ -12645,7 +12661,7 @@
       </c>
       <c r="AI93" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ93" t="inlineStr"/>
@@ -12729,7 +12745,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Printing and recorded media</t>
+          <t>Impresión y medios grabados</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -12792,7 +12808,7 @@
       <c r="AH94" t="inlineStr"/>
       <c r="AI94" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ94" t="inlineStr"/>
@@ -12856,7 +12872,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Cleaning products</t>
+          <t>Productos de limpieza</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -12915,7 +12931,7 @@
       <c r="AH95" t="inlineStr"/>
       <c r="AI95" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ95" t="inlineStr"/>
@@ -13062,7 +13078,7 @@
       <c r="AH96" t="inlineStr"/>
       <c r="AI96" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ96" t="inlineStr"/>
@@ -13189,7 +13205,7 @@
       <c r="AH97" t="inlineStr"/>
       <c r="AI97" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ97" t="inlineStr"/>
@@ -13308,7 +13324,7 @@
       <c r="AH98" t="inlineStr"/>
       <c r="AI98" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ98" t="inlineStr"/>
@@ -13443,7 +13459,7 @@
       <c r="AH99" t="inlineStr"/>
       <c r="AI99" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ99" t="inlineStr"/>
@@ -13554,7 +13570,7 @@
       <c r="AH100" t="inlineStr"/>
       <c r="AI100" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ100" t="inlineStr"/>
@@ -13681,7 +13697,7 @@
       <c r="AH101" t="inlineStr"/>
       <c r="AI101" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ101" t="inlineStr"/>
@@ -13913,7 +13929,7 @@
       <c r="AH103" t="inlineStr"/>
       <c r="AI103" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ103" t="inlineStr"/>
@@ -14044,7 +14060,7 @@
       <c r="AH104" t="inlineStr"/>
       <c r="AI104" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ104" t="inlineStr"/>
@@ -14116,7 +14132,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Remediation and other waste management</t>
+          <t>Gestión de residuos</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -14187,7 +14203,7 @@
       <c r="AH105" t="inlineStr"/>
       <c r="AI105" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ105" t="inlineStr"/>
@@ -14318,7 +14334,7 @@
       <c r="AH106" t="inlineStr"/>
       <c r="AI106" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ106" t="inlineStr"/>
@@ -14558,7 +14574,7 @@
       <c r="AH108" t="inlineStr"/>
       <c r="AI108" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ108" t="inlineStr"/>
@@ -14705,7 +14721,7 @@
       <c r="AH109" t="inlineStr"/>
       <c r="AI109" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ109" t="inlineStr"/>
@@ -14836,7 +14852,7 @@
       <c r="AH110" t="inlineStr"/>
       <c r="AI110" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ110" t="inlineStr"/>
@@ -14904,7 +14920,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Newspapers and magazines publishing</t>
+          <t>Edición de diarios y revistas</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -15086,7 +15102,7 @@
       <c r="AH112" t="inlineStr"/>
       <c r="AI112" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ112" t="inlineStr"/>
@@ -15217,7 +15233,7 @@
       <c r="AH113" t="inlineStr"/>
       <c r="AI113" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ113" t="inlineStr"/>
@@ -15340,11 +15356,19 @@
       <c r="AH114" t="inlineStr"/>
       <c r="AI114" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
-        </is>
-      </c>
-      <c r="AJ114" t="inlineStr"/>
-      <c r="AK114" t="inlineStr"/>
+          <t>Negativo</t>
+        </is>
+      </c>
+      <c r="AJ114" t="inlineStr">
+        <is>
+          <t>Pérdidas (2025-12): A septiembre de 2025 (nueve meses) la pérdida atribuible era de unos US$59,2 millones, con deterioro de activos cercano a US$80,6 millones ligado al cierre de campos en México y recambio varietal en Perú y China (Diario Frutícola, vía Italian Berry). | Cierre (2025-06): Su análisis razonado a junio de 2025 atribuye la pérdida de la temporada 24/25 (US$132,96 millones) principalmente a un deterioro de US$134,22 millones asociado al cierre de operaciones agrícolas en México. | Pérdidas (2025): El consolidado de Hortifrut S.A. registró una pérdida atribuible a la controladora de US$45,46 millones en 2024 y de US$77,73 millones en 2025, según su análisis razonado de diciembre de 2025.</t>
+        </is>
+      </c>
+      <c r="AK114" t="inlineStr">
+        <is>
+          <t>Las cifras son del consolidado Hortifrut S.A. (matriz); la ficha B corresponde a Hortifrut Chile, cuyas cuentas propias no se encontraron. Hay recuperación de ingresos: US$701 millones a junio de 2026, un 10,24% más que a junio de 2025 (análisis razonado de junio de 2026). Una segunda búsqueda no confirmó por separado la cifra anual de US$77,73 millones; conviene contrastarla con el documento original.</t>
+        </is>
+      </c>
       <c r="AL114" t="inlineStr"/>
       <c r="AM114" t="inlineStr"/>
       <c r="AN114" t="inlineStr"/>
@@ -15469,7 +15493,7 @@
       <c r="AH115" t="inlineStr"/>
       <c r="AI115" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ115" t="inlineStr"/>
@@ -15574,7 +15598,7 @@
       <c r="AH116" t="inlineStr"/>
       <c r="AI116" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ116" t="inlineStr"/>
@@ -15697,7 +15721,7 @@
       <c r="AH117" t="inlineStr"/>
       <c r="AI117" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ117" t="inlineStr"/>
@@ -15824,7 +15848,7 @@
       <c r="AH118" t="inlineStr"/>
       <c r="AI118" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ118" t="inlineStr"/>
@@ -15951,7 +15975,7 @@
       <c r="AH119" t="inlineStr"/>
       <c r="AI119" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ119" t="inlineStr"/>
@@ -16086,7 +16110,7 @@
       </c>
       <c r="AI120" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ120" t="inlineStr"/>
@@ -16233,7 +16257,7 @@
       </c>
       <c r="AI121" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ121" t="inlineStr"/>
@@ -16400,7 +16424,7 @@
       </c>
       <c r="AI122" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ122" t="inlineStr"/>
@@ -16660,7 +16684,7 @@
       </c>
       <c r="AI124" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ124" t="inlineStr"/>
@@ -16793,7 +16817,7 @@
       <c r="AH125" t="inlineStr"/>
       <c r="AI125" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ125" t="inlineStr"/>
@@ -16928,7 +16952,7 @@
       </c>
       <c r="AI126" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ126" t="inlineStr"/>
@@ -17071,7 +17095,7 @@
       <c r="AH127" t="inlineStr"/>
       <c r="AI127" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ127" t="inlineStr"/>
@@ -17210,7 +17234,7 @@
       </c>
       <c r="AI128" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ128" t="inlineStr"/>
@@ -17351,11 +17375,19 @@
       </c>
       <c r="AI129" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
-        </is>
-      </c>
-      <c r="AJ129" t="inlineStr"/>
-      <c r="AK129" t="inlineStr"/>
+          <t>Negativo</t>
+        </is>
+      </c>
+      <c r="AJ129" t="inlineStr">
+        <is>
+          <t>Rescate financiero (2025-03): Los family offices Wild Sur y Petra Luksic concretaron un aumento de capital de US$5 millones y quedaron con más del 60% de la propiedad; el fundador dejó el cargo de CEO. | Cierre (2024-09): Su CEO informó a inversionistas el inicio de un proceso de cierre por falta de financiamiento y pidió un cierre ordenado en vez de una liquidación judicial; fuentes cercanas señalaron que no había decisión final y que la carta buscaba presionar a los inversionistas.</t>
+        </is>
+      </c>
+      <c r="AK129" t="inlineStr">
+        <is>
+          <t>El cierre anunciado en septiembre de 2024 no se concretó: la empresa fue rescatada con capital fresco en marzo de 2025 (antes necesitaba con urgencia un aumento de capital de US$2 millones y dejó su casona-tienda de Puerto Varas). No se encontró información posterior a marzo de 2025.</t>
+        </is>
+      </c>
       <c r="AL129" t="inlineStr"/>
       <c r="AM129" t="inlineStr"/>
       <c r="AN129" t="inlineStr"/>
@@ -17476,7 +17508,7 @@
       <c r="AH130" t="inlineStr"/>
       <c r="AI130" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ130" t="inlineStr"/>
@@ -17601,7 +17633,7 @@
       <c r="AH131" t="inlineStr"/>
       <c r="AI131" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ131" t="inlineStr"/>
@@ -17732,7 +17764,7 @@
       <c r="AH132" t="inlineStr"/>
       <c r="AI132" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ132" t="inlineStr"/>
@@ -17859,7 +17891,7 @@
       <c r="AH133" t="inlineStr"/>
       <c r="AI133" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ133" t="inlineStr"/>
@@ -17978,7 +18010,7 @@
       <c r="AH134" t="inlineStr"/>
       <c r="AI134" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ134" t="inlineStr"/>
@@ -18099,7 +18131,7 @@
       <c r="AH135" t="inlineStr"/>
       <c r="AI135" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ135" t="inlineStr"/>
@@ -18226,7 +18258,7 @@
       <c r="AH136" t="inlineStr"/>
       <c r="AI136" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ136" t="inlineStr"/>
@@ -18357,7 +18389,7 @@
       <c r="AH137" t="inlineStr"/>
       <c r="AI137" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ137" t="inlineStr"/>
@@ -18488,7 +18520,7 @@
       <c r="AH138" t="inlineStr"/>
       <c r="AI138" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ138" t="inlineStr"/>
@@ -18623,7 +18655,7 @@
       <c r="AH139" t="inlineStr"/>
       <c r="AI139" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ139" t="inlineStr"/>
@@ -18869,7 +18901,7 @@
       <c r="AH141" t="inlineStr"/>
       <c r="AI141" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ141" t="inlineStr"/>
@@ -19000,7 +19032,7 @@
       <c r="AH142" t="inlineStr"/>
       <c r="AI142" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ142" t="inlineStr"/>
@@ -19262,7 +19294,7 @@
       <c r="AH144" t="inlineStr"/>
       <c r="AI144" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ144" t="inlineStr"/>
@@ -19381,7 +19413,7 @@
       <c r="AH145" t="inlineStr"/>
       <c r="AI145" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ145" t="inlineStr"/>
@@ -19494,7 +19526,7 @@
       <c r="AH146" t="inlineStr"/>
       <c r="AI146" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ146" t="inlineStr"/>
@@ -19740,7 +19772,7 @@
       <c r="AH148" t="inlineStr"/>
       <c r="AI148" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ148" t="inlineStr"/>
@@ -19857,7 +19889,7 @@
       <c r="AH149" t="inlineStr"/>
       <c r="AI149" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ149" t="inlineStr"/>
@@ -19996,7 +20028,7 @@
       <c r="AH150" t="inlineStr"/>
       <c r="AI150" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ150" t="inlineStr"/>
@@ -20107,7 +20139,7 @@
       <c r="AH151" t="inlineStr"/>
       <c r="AI151" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ151" t="inlineStr"/>
@@ -20458,7 +20490,7 @@
       <c r="AH154" t="inlineStr"/>
       <c r="AI154" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ154" t="inlineStr"/>
@@ -20585,7 +20617,7 @@
       <c r="AH155" t="inlineStr"/>
       <c r="AI155" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ155" t="inlineStr"/>
@@ -20716,7 +20748,7 @@
       <c r="AH156" t="inlineStr"/>
       <c r="AI156" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ156" t="inlineStr"/>
@@ -20841,7 +20873,7 @@
       <c r="AH157" t="inlineStr"/>
       <c r="AI157" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ157" t="inlineStr"/>
@@ -20962,7 +20994,7 @@
       <c r="AH158" t="inlineStr"/>
       <c r="AI158" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ158" t="inlineStr"/>
@@ -21077,7 +21109,7 @@
       <c r="AH159" t="inlineStr"/>
       <c r="AI159" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ159" t="inlineStr"/>
@@ -21309,7 +21341,7 @@
       <c r="AH161" t="inlineStr"/>
       <c r="AI161" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ161" t="inlineStr"/>
@@ -21436,7 +21468,7 @@
       <c r="AH162" t="inlineStr"/>
       <c r="AI162" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ162" t="inlineStr"/>
@@ -21567,7 +21599,7 @@
       <c r="AH163" t="inlineStr"/>
       <c r="AI163" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ163" t="inlineStr"/>
@@ -21821,7 +21853,7 @@
       <c r="AH165" t="inlineStr"/>
       <c r="AI165" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ165" t="inlineStr"/>
@@ -22071,7 +22103,7 @@
       <c r="AH167" t="inlineStr"/>
       <c r="AI167" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ167" t="inlineStr"/>
@@ -22202,7 +22234,7 @@
       <c r="AH168" t="inlineStr"/>
       <c r="AI168" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ168" t="inlineStr"/>
@@ -22337,7 +22369,7 @@
       <c r="AH169" t="inlineStr"/>
       <c r="AI169" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ169" t="inlineStr"/>
@@ -22464,11 +22496,19 @@
       <c r="AH170" t="inlineStr"/>
       <c r="AI170" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
-        </is>
-      </c>
-      <c r="AJ170" t="inlineStr"/>
-      <c r="AK170" t="inlineStr"/>
+          <t>En observación</t>
+        </is>
+      </c>
+      <c r="AJ170" t="inlineStr">
+        <is>
+          <t>Pérdidas (2023): La Tercera reportó que la cadena de panaderías registró pérdidas de $764 millones en 2019 y de $1.395 millones en 2020, según una carta de despido citada en un juicio laboral. | Despidos (2023): Según el mismo artículo, la empresa despidió a 187 trabajadores entre octubre de 2019 y 2023, justificando los despidos ante tribunales como ajuste de gastos operacionales al nivel real de ingresos.</t>
+        </is>
+      </c>
+      <c r="AK170" t="inlineStr">
+        <is>
+          <t>Situación recuperada según el mismo medio: sus estados financieros muestran utilidades en 2021 y 2022 (2022: $1.350 millones) y la empresa cuestionó los reportes de pérdidas de esos años, pese a que el titular habla de cuatro años de pérdidas. La fecha del artículo (2023) se infirió del contenido; no se encontró información posterior (2024-2026) sobre cierres, despidos o resultados. Revisión: Las pérdidas reportadas corresponden a 2019 y 2020; según el mismo medio, sus estados financieros muestran utilidades en 2021 y 2022 ($1.350 millones en 2022). No se encontró información posterior.</t>
+        </is>
+      </c>
       <c r="AL170" t="inlineStr"/>
       <c r="AM170" t="inlineStr"/>
       <c r="AN170" t="inlineStr"/>
@@ -22583,7 +22623,7 @@
       <c r="AH171" t="inlineStr"/>
       <c r="AI171" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ171" t="inlineStr"/>
@@ -22694,7 +22734,7 @@
       <c r="AH172" t="inlineStr"/>
       <c r="AI172" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ172" t="inlineStr"/>
@@ -22825,7 +22865,7 @@
       <c r="AH173" t="inlineStr"/>
       <c r="AI173" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ173" t="inlineStr"/>
@@ -22952,7 +22992,7 @@
       <c r="AH174" t="inlineStr"/>
       <c r="AI174" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ174" t="inlineStr"/>
@@ -23016,7 +23056,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>Technology-based support services</t>
+          <t>Servicios de soporte tecnológico</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
@@ -23176,7 +23216,7 @@
       <c r="AH176" t="inlineStr"/>
       <c r="AI176" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ176" t="inlineStr"/>
@@ -23404,7 +23444,7 @@
       <c r="AH178" t="inlineStr"/>
       <c r="AI178" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ178" t="inlineStr"/>
@@ -23583,7 +23623,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>Software publishing and SaaS</t>
+          <t>Software y plataformas SaaS</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
@@ -23642,7 +23682,7 @@
       <c r="AH180" t="inlineStr"/>
       <c r="AI180" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ180" t="inlineStr"/>
@@ -23710,7 +23750,7 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>Waste treatment and disposal</t>
+          <t>Tratamiento de residuos</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
@@ -23785,7 +23825,7 @@
       <c r="AH181" t="inlineStr"/>
       <c r="AI181" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ181" t="inlineStr"/>
@@ -23912,7 +23952,7 @@
       <c r="AH182" t="inlineStr"/>
       <c r="AI182" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ182" t="inlineStr"/>
@@ -24039,7 +24079,7 @@
       <c r="AH183" t="inlineStr"/>
       <c r="AI183" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ183" t="inlineStr"/>
@@ -24156,7 +24196,7 @@
       <c r="AH184" t="inlineStr"/>
       <c r="AI184" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ184" t="inlineStr"/>
@@ -24271,7 +24311,7 @@
       <c r="AH185" t="inlineStr"/>
       <c r="AI185" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ185" t="inlineStr"/>
@@ -24529,7 +24569,7 @@
       <c r="AH187" t="inlineStr"/>
       <c r="AI187" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ187" t="inlineStr"/>
@@ -24648,7 +24688,7 @@
       <c r="AH188" t="inlineStr"/>
       <c r="AI188" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ188" t="inlineStr"/>
@@ -24779,7 +24819,7 @@
       <c r="AH189" t="inlineStr"/>
       <c r="AI189" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ189" t="inlineStr"/>
@@ -24902,7 +24942,7 @@
       <c r="AH190" t="inlineStr"/>
       <c r="AI190" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ190" t="inlineStr"/>
@@ -24970,7 +25010,7 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>Computers and electronics</t>
+          <t>Computadores y electrónica</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
@@ -25033,7 +25073,7 @@
       <c r="AH191" t="inlineStr"/>
       <c r="AI191" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ191" t="inlineStr"/>
@@ -25396,7 +25436,7 @@
       <c r="AH194" t="inlineStr"/>
       <c r="AI194" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ194" t="inlineStr"/>
@@ -25527,7 +25567,7 @@
       <c r="AH195" t="inlineStr"/>
       <c r="AI195" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ195" t="inlineStr"/>
@@ -25595,7 +25635,7 @@
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>Other professional, scientific and technical activities</t>
+          <t>Otros servicios profesionales y científicos</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
@@ -25666,7 +25706,7 @@
       <c r="AH196" t="inlineStr"/>
       <c r="AI196" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ196" t="inlineStr"/>
@@ -25797,7 +25837,7 @@
       <c r="AH197" t="inlineStr"/>
       <c r="AI197" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ197" t="inlineStr"/>
@@ -25914,7 +25954,7 @@
       <c r="AH198" t="inlineStr"/>
       <c r="AI198" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ198" t="inlineStr"/>
@@ -26041,7 +26081,7 @@
       <c r="AH199" t="inlineStr"/>
       <c r="AI199" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ199" t="inlineStr"/>
@@ -26168,7 +26208,7 @@
       <c r="AH200" t="inlineStr"/>
       <c r="AI200" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ200" t="inlineStr"/>
@@ -26291,7 +26331,7 @@
       <c r="AH201" t="inlineStr"/>
       <c r="AI201" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ201" t="inlineStr"/>
@@ -26408,7 +26448,7 @@
       <c r="AH202" t="inlineStr"/>
       <c r="AI202" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ202" t="inlineStr"/>
@@ -26531,11 +26571,19 @@
       <c r="AH203" t="inlineStr"/>
       <c r="AI203" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
-        </is>
-      </c>
-      <c r="AJ203" t="inlineStr"/>
-      <c r="AK203" t="inlineStr"/>
+          <t>Negativo</t>
+        </is>
+      </c>
+      <c r="AJ203" t="inlineStr">
+        <is>
+          <t>Cierre (2026-09): Reportes de prensa señalan que vendió sus operaciones de Argentina y Uruguay a Molinos Río de la Plata, vendió Brasil al grupo Ferrara y cerró su oficina de México (hacia marzo de 2026, sin comprador y sin comunicado oficial). | Despidos (2026-09): Según Emol (citando a Diario Financiero), su plantilla pasó de un máximo de más de 300 personas a una cifra que hoy no superaría las 100. | Pérdidas (2026-09): Meganoticias informa que su operación en Chile sigue con resultados negativos y que tiene hasta fines de 2026 para demostrar que puede alcanzar la rentabilidad. | Despidos (2026-07): Desvinculó a 16 personas en Chile y EE.UU. (6 de I+D, 5 del equipo culinario, 4 de marketing y 1 de otras áreas de IA); la empresa confirmó las salidas sin detallar razones. | Despidos (2025-02): Cerró su oficina en Nueva York, encargó a Kraft Heinz la venta de sus productos en EE.UU. y Canadá y despidió a cerca del 11% de su plantilla para reducir costos (Bloomberg, citado por Emol).</t>
+        </is>
+      </c>
+      <c r="AK203" t="inlineStr">
+        <is>
+          <t>No hay declaración de insolvencia ni procedimiento concursal: la empresa sigue operando y se repliega hacia su negocio de IA (NotCo AI) y la rentabilidad en Chile; las salidas de países se describen como ventas o cierres de oficinas, no como liquidación. Ingresos 2025 estimados en cerca de US$70 millones (PitchBook, citado por Diario Financiero). Es el caso de mayor deterioro entre las startups revisadas, sin llegar al nivel crítico.</t>
+        </is>
+      </c>
       <c r="AL203" t="inlineStr"/>
       <c r="AM203" t="inlineStr"/>
       <c r="AN203" t="inlineStr"/>
@@ -26662,7 +26710,7 @@
       <c r="AH204" t="inlineStr"/>
       <c r="AI204" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ204" t="inlineStr"/>
@@ -26789,7 +26837,7 @@
       <c r="AH205" t="inlineStr"/>
       <c r="AI205" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ205" t="inlineStr"/>
@@ -26908,7 +26956,7 @@
       <c r="AH206" t="inlineStr"/>
       <c r="AI206" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ206" t="inlineStr"/>
@@ -27043,7 +27091,7 @@
       <c r="AH207" t="inlineStr"/>
       <c r="AI207" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ207" t="inlineStr"/>
@@ -27170,7 +27218,7 @@
       <c r="AH208" t="inlineStr"/>
       <c r="AI208" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ208" t="inlineStr"/>
@@ -27295,7 +27343,7 @@
       <c r="AH209" t="inlineStr"/>
       <c r="AI209" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ209" t="inlineStr"/>
@@ -27434,7 +27482,7 @@
       <c r="AH210" t="inlineStr"/>
       <c r="AI210" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ210" t="inlineStr"/>
@@ -27547,7 +27595,7 @@
       <c r="AH211" t="inlineStr"/>
       <c r="AI211" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ211" t="inlineStr"/>
@@ -27793,7 +27841,7 @@
       <c r="AH213" t="inlineStr"/>
       <c r="AI213" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ213" t="inlineStr"/>
@@ -27940,11 +27988,19 @@
       <c r="AH214" t="inlineStr"/>
       <c r="AI214" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
-        </is>
-      </c>
-      <c r="AJ214" t="inlineStr"/>
-      <c r="AK214" t="inlineStr"/>
+          <t>En observación</t>
+        </is>
+      </c>
+      <c r="AJ214" t="inlineStr">
+        <is>
+          <t>Caída de ventas (2026-05): En el primer trimestre de 2026 las ventas cayeron 7,8% (a $192.613 millones) y la utilidad atribuible bajó 36,3% (a $8.779 millones). | Caída de ventas (2026): En el primer semestre de 2026 las ventas retrocedieron 6,2% (a $425.895 millones) y las ganancias cayeron 14% (a $28.186 millones), por menores ventas en EE.UU. y en algunos mercados de exportación.</t>
+        </is>
+      </c>
+      <c r="AK214" t="inlineStr">
+        <is>
+          <t>Sigue siendo rentable y fue una de las dos viñas reportantes a la CMF con utilidades en 2025 (utilidad 2025 de $67.220 millones, -13,1%; ingresos 2025 +1,7%). En el segundo trimestre de 2026 la utilidad subió 2,1% y la compañía proyecta crecimiento de un dígito para 2026. Señal negativa moderada, sin indicios de insolvencia.</t>
+        </is>
+      </c>
       <c r="AL214" t="inlineStr"/>
       <c r="AM214" t="inlineStr"/>
       <c r="AN214" t="inlineStr"/>
@@ -28008,7 +28064,7 @@
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>Agricultural support and post-harvest</t>
+          <t>Servicios agrícolas y poscosecha</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
@@ -28065,11 +28121,19 @@
       <c r="AH215" t="inlineStr"/>
       <c r="AI215" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
-        </is>
-      </c>
-      <c r="AJ215" t="inlineStr"/>
-      <c r="AK215" t="inlineStr"/>
+          <t>Negativo</t>
+        </is>
+      </c>
+      <c r="AJ215" t="inlineStr">
+        <is>
+          <t>Pérdidas (2025): Cerró 2025 con pérdidas (reportes citan unos US$0,47 millones, con ingresos -5,3%) tras una pérdida cercana a US$4,75 millones en 2024; es una de las cuatro viñas con pérdidas entre las seis que reportan a la CMF.</t>
+        </is>
+      </c>
+      <c r="AK215" t="inlineStr">
+        <is>
+          <t>La pérdida se redujo de 2024 a 2025. Contexto de caída del consumo mundial de vino; en el primer semestre de 2026 las seis viñas CMF mostraron caídas de ingresos (Emol, 2026-08). Las cifras exactas provienen de resúmenes de prensa y conviene contrastarlas con los estados financieros CMF.</t>
+        </is>
+      </c>
       <c r="AL215" t="inlineStr"/>
       <c r="AM215" t="inlineStr"/>
       <c r="AN215" t="inlineStr"/>
@@ -28184,7 +28248,7 @@
       <c r="AH216" t="inlineStr"/>
       <c r="AI216" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ216" t="inlineStr"/>
@@ -28311,7 +28375,7 @@
       <c r="AH217" t="inlineStr"/>
       <c r="AI217" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ217" t="inlineStr"/>
@@ -28438,11 +28502,19 @@
       <c r="AH218" t="inlineStr"/>
       <c r="AI218" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
-        </is>
-      </c>
-      <c r="AJ218" t="inlineStr"/>
-      <c r="AK218" t="inlineStr"/>
+          <t>Negativo</t>
+        </is>
+      </c>
+      <c r="AJ218" t="inlineStr">
+        <is>
+          <t>Pérdidas (2026-08): En el primer semestre de 2026 facturó 12,86% menos y registró pérdidas de $318 millones, frente a una ganancia de $684 millones en igual período de 2025. | Pérdidas (2026-03): Cerró el ejercicio 2025 con una pérdida de $195,7 millones y con ingresos 3,19% menores ($28.716 millones), según Vinetur sobre estados financieros presentados a la CMF.</t>
+        </is>
+      </c>
+      <c r="AK218" t="inlineStr">
+        <is>
+          <t>Forma parte de las viñas con pérdidas en un contexto de caída del consumo mundial de vino (solo dos de las seis viñas que reportan a la CMF cerraron 2025 con utilidades). Según sus estados financieros, en 2024 el directorio aprobó el proceso de venta del Fundo Totihue. El resultado anual 2025 de Emiliana no se verificó de forma directa.</t>
+        </is>
+      </c>
       <c r="AL218" t="inlineStr"/>
       <c r="AM218" t="inlineStr"/>
       <c r="AN218" t="inlineStr"/>
@@ -28577,7 +28649,7 @@
       <c r="AH219" t="inlineStr"/>
       <c r="AI219" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ219" t="inlineStr"/>
@@ -28708,7 +28780,7 @@
       <c r="AH220" t="inlineStr"/>
       <c r="AI220" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ220" t="inlineStr"/>
@@ -28821,7 +28893,7 @@
       <c r="AH221" t="inlineStr"/>
       <c r="AI221" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ221" t="inlineStr"/>
@@ -28889,7 +28961,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>Cleaning products</t>
+          <t>Productos de limpieza</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
@@ -28948,7 +29020,7 @@
       <c r="AH222" t="inlineStr"/>
       <c r="AI222" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ222" t="inlineStr"/>
@@ -29091,7 +29163,7 @@
       <c r="AH223" t="inlineStr"/>
       <c r="AI223" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ223" t="inlineStr"/>
@@ -29218,7 +29290,7 @@
       <c r="AH224" t="inlineStr"/>
       <c r="AI224" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ224" t="inlineStr"/>
@@ -29353,7 +29425,7 @@
       <c r="AH225" t="inlineStr"/>
       <c r="AI225" t="inlineStr">
         <is>
-          <t>Sin revisar</t>
+          <t>Sin señales públicas</t>
         </is>
       </c>
       <c r="AJ225" t="inlineStr"/>

</xml_diff>